<commit_message>
some work on VT7 and add Murky
</commit_message>
<xml_diff>
--- a/__docs/RoadMap.xlsx
+++ b/__docs/RoadMap.xlsx
@@ -8,15 +8,16 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Dev\exchange\RichLaughter3\__docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6DE72FD0-D8B3-4A83-8C9C-00DE45FE4412}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E2CD221D-DEAA-483A-A62C-1D97C11664DC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Тезисы" sheetId="1" r:id="rId1"/>
     <sheet name="Древо" sheetId="2" r:id="rId2"/>
     <sheet name="Задачи" sheetId="3" r:id="rId3"/>
     <sheet name="Стратегии" sheetId="4" r:id="rId4"/>
+    <sheet name="Лист1" sheetId="5" r:id="rId5"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -28,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="36">
   <si>
     <t>RL3 - это продолжение RL1</t>
   </si>
@@ -101,6 +102,42 @@
   <si>
     <t>Заменить pag на pdi в VT7</t>
   </si>
+  <si>
+    <t>Название</t>
+  </si>
+  <si>
+    <t>Дата</t>
+  </si>
+  <si>
+    <t>К</t>
+  </si>
+  <si>
+    <t>Описание</t>
+  </si>
+  <si>
+    <t>ЦАТ</t>
+  </si>
+  <si>
+    <t>PEG30_RAYNOR</t>
+  </si>
+  <si>
+    <t>PEG30_MURKY</t>
+  </si>
+  <si>
+    <t>Адапт. PTA30_RAYNOR</t>
+  </si>
+  <si>
+    <t>Сборщик спреда на базе PTA30</t>
+  </si>
+  <si>
+    <t>PEG2_DDCrWork</t>
+  </si>
+  <si>
+    <t>Адапт. PTA2_DCCrWork</t>
+  </si>
+  <si>
+    <t>Новый мультистратеговый трейдер для Cscalp</t>
+  </si>
 </sst>
 </file>
 
@@ -141,7 +178,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -150,10 +187,13 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Обычный" xfId="0" builtinId="0"/>
@@ -487,7 +527,7 @@
       </c>
     </row>
     <row r="3" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B3" s="4" t="s">
+      <c r="B3" s="5" t="s">
         <v>3</v>
       </c>
       <c r="C3" s="2" t="s">
@@ -495,13 +535,13 @@
       </c>
     </row>
     <row r="4" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B4" s="4"/>
+      <c r="B4" s="5"/>
       <c r="C4" s="2" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="5" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B5" s="4" t="s">
+      <c r="B5" s="5" t="s">
         <v>4</v>
       </c>
       <c r="C5" s="2" t="s">
@@ -509,43 +549,43 @@
       </c>
     </row>
     <row r="6" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B6" s="4"/>
+      <c r="B6" s="5"/>
       <c r="C6" s="2" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="7" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B7" s="4"/>
+      <c r="B7" s="5"/>
       <c r="C7" s="2" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="8" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B8" s="4"/>
+      <c r="B8" s="5"/>
       <c r="C8" s="2" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="9" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B9" s="4"/>
+      <c r="B9" s="5"/>
       <c r="C9" s="2" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="10" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B10" s="4"/>
+      <c r="B10" s="5"/>
       <c r="C10" s="2" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="11" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B11" s="4"/>
+      <c r="B11" s="5"/>
       <c r="C11" s="2" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="12" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B12" s="4"/>
+      <c r="B12" s="5"/>
       <c r="C12" s="2" t="s">
         <v>17</v>
       </c>
@@ -593,7 +633,7 @@
       <c r="A2">
         <v>1</v>
       </c>
-      <c r="B2" s="5" t="s">
+      <c r="B2" s="4" t="s">
         <v>22</v>
       </c>
       <c r="C2" s="3">
@@ -3661,4 +3701,2068 @@
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AD38F229-6CC0-4A34-802C-B9D336FEB24E}">
+  <dimension ref="A1:E398"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="2" max="2" width="21.5703125" customWidth="1"/>
+    <col min="3" max="3" width="14" customWidth="1"/>
+    <col min="4" max="4" width="21.5703125" customWidth="1"/>
+    <col min="5" max="5" width="44.85546875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="B1" t="s">
+        <v>24</v>
+      </c>
+      <c r="C1" t="s">
+        <v>25</v>
+      </c>
+      <c r="D1" t="s">
+        <v>26</v>
+      </c>
+      <c r="E1" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2">
+        <v>1</v>
+      </c>
+      <c r="B2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C2" s="3">
+        <v>46230</v>
+      </c>
+      <c r="D2" t="s">
+        <v>28</v>
+      </c>
+      <c r="E2" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A3">
+        <v>2</v>
+      </c>
+      <c r="B3" t="s">
+        <v>33</v>
+      </c>
+      <c r="C3" s="3">
+        <v>46233</v>
+      </c>
+      <c r="D3" t="s">
+        <v>12</v>
+      </c>
+      <c r="E3" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A4">
+        <v>3</v>
+      </c>
+      <c r="B4" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="C4" s="3">
+        <v>46237</v>
+      </c>
+      <c r="D4" t="s">
+        <v>12</v>
+      </c>
+      <c r="E4" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A5">
+        <v>4</v>
+      </c>
+      <c r="B5" t="s">
+        <v>30</v>
+      </c>
+      <c r="C5" s="3">
+        <v>46238</v>
+      </c>
+      <c r="D5" t="s">
+        <v>12</v>
+      </c>
+      <c r="E5" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A6">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A7">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A8">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A9">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A10">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A11">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A12">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A13">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A14">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A15">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A16">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="17" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A17">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="18" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A18">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="19" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A19">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="20" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A20">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="21" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A21">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="22" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A22">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="23" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A23">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="24" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A24">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="25" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A25">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="26" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A26">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="27" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A27">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="28" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A28">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="29" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A29">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="30" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A30">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="31" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A31">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="32" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A32">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="33" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A33">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="34" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A34">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="35" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A35">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="36" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A36">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="37" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A37">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="38" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A38">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="39" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A39">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="40" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A40">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="41" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A41">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="42" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A42">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="43" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A43">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="44" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A44">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="45" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A45">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="46" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A46">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="47" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A47">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="48" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A48">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="49" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A49">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="50" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A50">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="51" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A51">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="52" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A52">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="53" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A53">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="54" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A54">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="55" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A55">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="56" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A56">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="57" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A57">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="58" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A58">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="59" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A59">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="60" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A60">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="61" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A61">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="62" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A62">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="63" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A63">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="64" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A64">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="65" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A65">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="66" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A66">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="67" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A67">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="68" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A68">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="69" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A69">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="70" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A70">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="71" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A71">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="72" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A72">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="73" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A73">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="74" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A74">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="75" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A75">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="76" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A76">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="77" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A77">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="78" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A78">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="79" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A79">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="80" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A80">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="81" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A81">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="82" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A82">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="83" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A83">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="84" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A84">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="85" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A85">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="86" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A86">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="87" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A87">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="88" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A88">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="89" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A89">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="90" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A90">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="91" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A91">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="92" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A92">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="93" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A93">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="94" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A94">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="95" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A95">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="96" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A96">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="97" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A97">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="98" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A98">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="99" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A99">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="100" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A100">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="101" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A101">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="102" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A102">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="103" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A103">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="104" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A104">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="105" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A105">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="106" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A106">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="107" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A107">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="108" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A108">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="109" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A109">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="110" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A110">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="111" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A111">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="112" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A112">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="113" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A113">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="114" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A114">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="115" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A115">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="116" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A116">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="117" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A117">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="118" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A118">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="119" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A119">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="120" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A120">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="121" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A121">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="122" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A122">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="123" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A123">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="124" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A124">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="125" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A125">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="126" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A126">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="127" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A127">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="128" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A128">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="129" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A129">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="130" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A130">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="131" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A131">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="132" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A132">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="133" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A133">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="134" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A134">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="135" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A135">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="136" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A136">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="137" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A137">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="138" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A138">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="139" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A139">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="140" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A140">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="141" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A141">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="142" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A142">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="143" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A143">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="144" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A144">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="145" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A145">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="146" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A146">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="147" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A147">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="148" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A148">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="149" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A149">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="150" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A150">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="151" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A151">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="152" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A152">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="153" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A153">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="154" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A154">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="155" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A155">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="156" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A156">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="157" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A157">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="158" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A158">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="159" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A159">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="160" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A160">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="161" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A161">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="162" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A162">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="163" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A163">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="164" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A164">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="165" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A165">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="166" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A166">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="167" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A167">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="168" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A168">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="169" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A169">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="170" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A170">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="171" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A171">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="172" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A172">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="173" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A173">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="174" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A174">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="175" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A175">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="176" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A176">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="177" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A177">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="178" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A178">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="179" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A179">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="180" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A180">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="181" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A181">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="182" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A182">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="183" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A183">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="184" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A184">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="185" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A185">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="186" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A186">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="187" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A187">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="188" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A188">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="189" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A189">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="190" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A190">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="191" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A191">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="192" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A192">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="193" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A193">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="194" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A194">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="195" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A195">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="196" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A196">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="197" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A197">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="198" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A198">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="199" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A199">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="200" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A200">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="201" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A201">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="202" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A202">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="203" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A203">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="204" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A204">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="205" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A205">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="206" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A206">
+        <v>205</v>
+      </c>
+    </row>
+    <row r="207" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A207">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="208" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A208">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="209" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A209">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="210" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A210">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="211" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A211">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="212" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A212">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="213" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A213">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="214" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A214">
+        <v>213</v>
+      </c>
+    </row>
+    <row r="215" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A215">
+        <v>214</v>
+      </c>
+    </row>
+    <row r="216" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A216">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="217" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A217">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="218" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A218">
+        <v>217</v>
+      </c>
+    </row>
+    <row r="219" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A219">
+        <v>218</v>
+      </c>
+    </row>
+    <row r="220" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A220">
+        <v>219</v>
+      </c>
+    </row>
+    <row r="221" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A221">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="222" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A222">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="223" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A223">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="224" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A224">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="225" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A225">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="226" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A226">
+        <v>225</v>
+      </c>
+    </row>
+    <row r="227" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A227">
+        <v>226</v>
+      </c>
+    </row>
+    <row r="228" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A228">
+        <v>227</v>
+      </c>
+    </row>
+    <row r="229" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A229">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="230" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A230">
+        <v>229</v>
+      </c>
+    </row>
+    <row r="231" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A231">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="232" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A232">
+        <v>231</v>
+      </c>
+    </row>
+    <row r="233" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A233">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="234" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A234">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="235" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A235">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="236" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A236">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="237" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A237">
+        <v>236</v>
+      </c>
+    </row>
+    <row r="238" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A238">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="239" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A239">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="240" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A240">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="241" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A241">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="242" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A242">
+        <v>241</v>
+      </c>
+    </row>
+    <row r="243" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A243">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="244" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A244">
+        <v>243</v>
+      </c>
+    </row>
+    <row r="245" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A245">
+        <v>244</v>
+      </c>
+    </row>
+    <row r="246" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A246">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="247" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A247">
+        <v>246</v>
+      </c>
+    </row>
+    <row r="248" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A248">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="249" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A249">
+        <v>248</v>
+      </c>
+    </row>
+    <row r="250" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A250">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="251" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A251">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="252" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A252">
+        <v>251</v>
+      </c>
+    </row>
+    <row r="253" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A253">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="254" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A254">
+        <v>253</v>
+      </c>
+    </row>
+    <row r="255" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A255">
+        <v>254</v>
+      </c>
+    </row>
+    <row r="256" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A256">
+        <v>255</v>
+      </c>
+    </row>
+    <row r="257" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A257">
+        <v>256</v>
+      </c>
+    </row>
+    <row r="258" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A258">
+        <v>257</v>
+      </c>
+    </row>
+    <row r="259" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A259">
+        <v>258</v>
+      </c>
+    </row>
+    <row r="260" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A260">
+        <v>259</v>
+      </c>
+    </row>
+    <row r="261" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A261">
+        <v>260</v>
+      </c>
+    </row>
+    <row r="262" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A262">
+        <v>261</v>
+      </c>
+    </row>
+    <row r="263" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A263">
+        <v>262</v>
+      </c>
+    </row>
+    <row r="264" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A264">
+        <v>263</v>
+      </c>
+    </row>
+    <row r="265" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A265">
+        <v>264</v>
+      </c>
+    </row>
+    <row r="266" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A266">
+        <v>265</v>
+      </c>
+    </row>
+    <row r="267" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A267">
+        <v>266</v>
+      </c>
+    </row>
+    <row r="268" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A268">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="269" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A269">
+        <v>268</v>
+      </c>
+    </row>
+    <row r="270" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A270">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="271" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A271">
+        <v>270</v>
+      </c>
+    </row>
+    <row r="272" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A272">
+        <v>271</v>
+      </c>
+    </row>
+    <row r="273" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A273">
+        <v>272</v>
+      </c>
+    </row>
+    <row r="274" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A274">
+        <v>273</v>
+      </c>
+    </row>
+    <row r="275" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A275">
+        <v>274</v>
+      </c>
+    </row>
+    <row r="276" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A276">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="277" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A277">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="278" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A278">
+        <v>277</v>
+      </c>
+    </row>
+    <row r="279" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A279">
+        <v>278</v>
+      </c>
+    </row>
+    <row r="280" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A280">
+        <v>279</v>
+      </c>
+    </row>
+    <row r="281" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A281">
+        <v>280</v>
+      </c>
+    </row>
+    <row r="282" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A282">
+        <v>281</v>
+      </c>
+    </row>
+    <row r="283" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A283">
+        <v>282</v>
+      </c>
+    </row>
+    <row r="284" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A284">
+        <v>283</v>
+      </c>
+    </row>
+    <row r="285" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A285">
+        <v>284</v>
+      </c>
+    </row>
+    <row r="286" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A286">
+        <v>285</v>
+      </c>
+    </row>
+    <row r="287" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A287">
+        <v>286</v>
+      </c>
+    </row>
+    <row r="288" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A288">
+        <v>287</v>
+      </c>
+    </row>
+    <row r="289" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A289">
+        <v>288</v>
+      </c>
+    </row>
+    <row r="290" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A290">
+        <v>289</v>
+      </c>
+    </row>
+    <row r="291" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A291">
+        <v>290</v>
+      </c>
+    </row>
+    <row r="292" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A292">
+        <v>291</v>
+      </c>
+    </row>
+    <row r="293" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A293">
+        <v>292</v>
+      </c>
+    </row>
+    <row r="294" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A294">
+        <v>293</v>
+      </c>
+    </row>
+    <row r="295" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A295">
+        <v>294</v>
+      </c>
+    </row>
+    <row r="296" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A296">
+        <v>295</v>
+      </c>
+    </row>
+    <row r="297" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A297">
+        <v>296</v>
+      </c>
+    </row>
+    <row r="298" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A298">
+        <v>297</v>
+      </c>
+    </row>
+    <row r="299" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A299">
+        <v>298</v>
+      </c>
+    </row>
+    <row r="300" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A300">
+        <v>299</v>
+      </c>
+    </row>
+    <row r="301" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A301">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="302" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A302">
+        <v>301</v>
+      </c>
+    </row>
+    <row r="303" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A303">
+        <v>302</v>
+      </c>
+    </row>
+    <row r="304" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A304">
+        <v>303</v>
+      </c>
+    </row>
+    <row r="305" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A305">
+        <v>304</v>
+      </c>
+    </row>
+    <row r="306" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A306">
+        <v>305</v>
+      </c>
+    </row>
+    <row r="307" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A307">
+        <v>306</v>
+      </c>
+    </row>
+    <row r="308" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A308">
+        <v>307</v>
+      </c>
+    </row>
+    <row r="309" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A309">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="310" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A310">
+        <v>309</v>
+      </c>
+    </row>
+    <row r="311" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A311">
+        <v>310</v>
+      </c>
+    </row>
+    <row r="312" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A312">
+        <v>311</v>
+      </c>
+    </row>
+    <row r="313" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A313">
+        <v>312</v>
+      </c>
+    </row>
+    <row r="314" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A314">
+        <v>313</v>
+      </c>
+    </row>
+    <row r="315" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A315">
+        <v>314</v>
+      </c>
+    </row>
+    <row r="316" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A316">
+        <v>315</v>
+      </c>
+    </row>
+    <row r="317" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A317">
+        <v>316</v>
+      </c>
+    </row>
+    <row r="318" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A318">
+        <v>317</v>
+      </c>
+    </row>
+    <row r="319" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A319">
+        <v>318</v>
+      </c>
+    </row>
+    <row r="320" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A320">
+        <v>319</v>
+      </c>
+    </row>
+    <row r="321" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A321">
+        <v>320</v>
+      </c>
+    </row>
+    <row r="322" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A322">
+        <v>321</v>
+      </c>
+    </row>
+    <row r="323" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A323">
+        <v>322</v>
+      </c>
+    </row>
+    <row r="324" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A324">
+        <v>323</v>
+      </c>
+    </row>
+    <row r="325" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A325">
+        <v>324</v>
+      </c>
+    </row>
+    <row r="326" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A326">
+        <v>325</v>
+      </c>
+    </row>
+    <row r="327" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A327">
+        <v>326</v>
+      </c>
+    </row>
+    <row r="328" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A328">
+        <v>327</v>
+      </c>
+    </row>
+    <row r="329" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A329">
+        <v>328</v>
+      </c>
+    </row>
+    <row r="330" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A330">
+        <v>329</v>
+      </c>
+    </row>
+    <row r="331" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A331">
+        <v>330</v>
+      </c>
+    </row>
+    <row r="332" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A332">
+        <v>331</v>
+      </c>
+    </row>
+    <row r="333" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A333">
+        <v>332</v>
+      </c>
+    </row>
+    <row r="334" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A334">
+        <v>333</v>
+      </c>
+    </row>
+    <row r="335" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A335">
+        <v>334</v>
+      </c>
+    </row>
+    <row r="336" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A336">
+        <v>335</v>
+      </c>
+    </row>
+    <row r="337" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A337">
+        <v>336</v>
+      </c>
+    </row>
+    <row r="338" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A338">
+        <v>337</v>
+      </c>
+    </row>
+    <row r="339" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A339">
+        <v>338</v>
+      </c>
+    </row>
+    <row r="340" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A340">
+        <v>339</v>
+      </c>
+    </row>
+    <row r="341" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A341">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="342" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A342">
+        <v>341</v>
+      </c>
+    </row>
+    <row r="343" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A343">
+        <v>342</v>
+      </c>
+    </row>
+    <row r="344" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A344">
+        <v>343</v>
+      </c>
+    </row>
+    <row r="345" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A345">
+        <v>344</v>
+      </c>
+    </row>
+    <row r="346" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A346">
+        <v>345</v>
+      </c>
+    </row>
+    <row r="347" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A347">
+        <v>346</v>
+      </c>
+    </row>
+    <row r="348" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A348">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="349" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A349">
+        <v>348</v>
+      </c>
+    </row>
+    <row r="350" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A350">
+        <v>349</v>
+      </c>
+    </row>
+    <row r="351" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A351">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="352" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A352">
+        <v>351</v>
+      </c>
+    </row>
+    <row r="353" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A353">
+        <v>352</v>
+      </c>
+    </row>
+    <row r="354" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A354">
+        <v>353</v>
+      </c>
+    </row>
+    <row r="355" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A355">
+        <v>354</v>
+      </c>
+    </row>
+    <row r="356" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A356">
+        <v>355</v>
+      </c>
+    </row>
+    <row r="357" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A357">
+        <v>356</v>
+      </c>
+    </row>
+    <row r="358" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A358">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="359" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A359">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="360" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A360">
+        <v>359</v>
+      </c>
+    </row>
+    <row r="361" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A361">
+        <v>360</v>
+      </c>
+    </row>
+    <row r="362" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A362">
+        <v>361</v>
+      </c>
+    </row>
+    <row r="363" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A363">
+        <v>362</v>
+      </c>
+    </row>
+    <row r="364" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A364">
+        <v>363</v>
+      </c>
+    </row>
+    <row r="365" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A365">
+        <v>364</v>
+      </c>
+    </row>
+    <row r="366" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A366">
+        <v>365</v>
+      </c>
+    </row>
+    <row r="367" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A367">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="368" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A368">
+        <v>367</v>
+      </c>
+    </row>
+    <row r="369" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A369">
+        <v>368</v>
+      </c>
+    </row>
+    <row r="370" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A370">
+        <v>369</v>
+      </c>
+    </row>
+    <row r="371" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A371">
+        <v>370</v>
+      </c>
+    </row>
+    <row r="372" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A372">
+        <v>371</v>
+      </c>
+    </row>
+    <row r="373" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A373">
+        <v>372</v>
+      </c>
+    </row>
+    <row r="374" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A374">
+        <v>373</v>
+      </c>
+    </row>
+    <row r="375" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A375">
+        <v>374</v>
+      </c>
+    </row>
+    <row r="376" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A376">
+        <v>375</v>
+      </c>
+    </row>
+    <row r="377" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A377">
+        <v>376</v>
+      </c>
+    </row>
+    <row r="378" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A378">
+        <v>377</v>
+      </c>
+    </row>
+    <row r="379" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A379">
+        <v>378</v>
+      </c>
+    </row>
+    <row r="380" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A380">
+        <v>379</v>
+      </c>
+    </row>
+    <row r="381" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A381">
+        <v>380</v>
+      </c>
+    </row>
+    <row r="382" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A382">
+        <v>381</v>
+      </c>
+    </row>
+    <row r="383" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A383">
+        <v>382</v>
+      </c>
+    </row>
+    <row r="384" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A384">
+        <v>383</v>
+      </c>
+    </row>
+    <row r="385" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A385">
+        <v>384</v>
+      </c>
+    </row>
+    <row r="386" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A386">
+        <v>385</v>
+      </c>
+    </row>
+    <row r="387" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A387">
+        <v>386</v>
+      </c>
+    </row>
+    <row r="388" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A388">
+        <v>387</v>
+      </c>
+    </row>
+    <row r="389" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A389">
+        <v>388</v>
+      </c>
+    </row>
+    <row r="390" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A390">
+        <v>389</v>
+      </c>
+    </row>
+    <row r="391" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A391">
+        <v>390</v>
+      </c>
+    </row>
+    <row r="392" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A392">
+        <v>391</v>
+      </c>
+    </row>
+    <row r="393" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A393">
+        <v>392</v>
+      </c>
+    </row>
+    <row r="394" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A394">
+        <v>393</v>
+      </c>
+    </row>
+    <row r="395" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A395">
+        <v>394</v>
+      </c>
+    </row>
+    <row r="396" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A396">
+        <v>395</v>
+      </c>
+    </row>
+    <row r="397" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A397">
+        <v>396</v>
+      </c>
+    </row>
+    <row r="398" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A398">
+        <v>397</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
start work on testing
</commit_message>
<xml_diff>
--- a/__docs/RoadMap.xlsx
+++ b/__docs/RoadMap.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Dev\exchange\RichLaughter3\__docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E2CD221D-DEAA-483A-A62C-1D97C11664DC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4E30F83C-F071-4D7A-B44D-526A5949620A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -17,7 +17,7 @@
     <sheet name="Древо" sheetId="2" r:id="rId2"/>
     <sheet name="Задачи" sheetId="3" r:id="rId3"/>
     <sheet name="Стратегии" sheetId="4" r:id="rId4"/>
-    <sheet name="Лист1" sheetId="5" r:id="rId5"/>
+    <sheet name="ДрРоботов" sheetId="5" r:id="rId5"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="36">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="37">
   <si>
     <t>RL3 - это продолжение RL1</t>
   </si>
@@ -138,6 +138,9 @@
   <si>
     <t>Новый мультистратеговый трейдер для Cscalp</t>
   </si>
+  <si>
+    <t>Нельзя менять, pag делает скриншоты удобно</t>
+  </si>
 </sst>
 </file>
 
@@ -152,7 +155,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -162,6 +165,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC000"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -178,7 +187,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -189,11 +198,12 @@
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Обычный" xfId="0" builtinId="0"/>
@@ -527,7 +537,7 @@
       </c>
     </row>
     <row r="3" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B3" s="5" t="s">
+      <c r="B3" s="6" t="s">
         <v>3</v>
       </c>
       <c r="C3" s="2" t="s">
@@ -535,13 +545,13 @@
       </c>
     </row>
     <row r="4" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B4" s="5"/>
+      <c r="B4" s="6"/>
       <c r="C4" s="2" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="5" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B5" s="5" t="s">
+      <c r="B5" s="6" t="s">
         <v>4</v>
       </c>
       <c r="C5" s="2" t="s">
@@ -549,43 +559,43 @@
       </c>
     </row>
     <row r="6" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B6" s="5"/>
+      <c r="B6" s="6"/>
       <c r="C6" s="2" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="7" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B7" s="5"/>
+      <c r="B7" s="6"/>
       <c r="C7" s="2" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="8" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B8" s="5"/>
+      <c r="B8" s="6"/>
       <c r="C8" s="2" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="9" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B9" s="5"/>
+      <c r="B9" s="6"/>
       <c r="C9" s="2" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="10" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B10" s="5"/>
+      <c r="B10" s="6"/>
       <c r="C10" s="2" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="11" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B11" s="5"/>
+      <c r="B11" s="6"/>
       <c r="C11" s="2" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="12" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B12" s="5"/>
+      <c r="B12" s="6"/>
       <c r="C12" s="2" t="s">
         <v>17</v>
       </c>
@@ -610,7 +620,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9DBD1468-2D66-4691-A039-8F66EC21E445}">
-  <dimension ref="A1:D610"/>
+  <dimension ref="A1:E610"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="56" customWidth="1"/>
@@ -618,7 +628,7 @@
     <col min="4" max="4" width="18.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B1" s="1" t="s">
         <v>19</v>
       </c>
@@ -629,7 +639,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>1</v>
       </c>
@@ -643,78 +653,84 @@
         <v>46227</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>2</v>
       </c>
-      <c r="B3" t="s">
+      <c r="B3" s="7" t="s">
         <v>23</v>
       </c>
       <c r="C3" s="3">
         <v>46228</v>
       </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D3" s="3">
+        <v>46237</v>
+      </c>
+      <c r="E3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>3</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>4</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>5</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>6</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>7</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>8</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>9</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>10</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12">
         <v>11</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13">
         <v>12</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14">
         <v>13</v>
       </c>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15">
         <v>14</v>
       </c>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16">
         <v>15</v>
       </c>
@@ -3766,7 +3782,7 @@
       <c r="A4">
         <v>3</v>
       </c>
-      <c r="B4" s="6" t="s">
+      <c r="B4" s="5" t="s">
         <v>29</v>
       </c>
       <c r="C4" s="3">

</xml_diff>

<commit_message>
add first adapt startegies
</commit_message>
<xml_diff>
--- a/__docs/RoadMap.xlsx
+++ b/__docs/RoadMap.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Dev\exchange\RichLaughter3\__docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F96AA9FF-D9DF-4F76-917A-0EA66C4A14AA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{82418D2F-12F3-41BD-8FCA-F1FF8B44FEF2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -18,18 +18,28 @@
     <sheet name="Задачи" sheetId="3" r:id="rId3"/>
     <sheet name="Стратегии" sheetId="4" r:id="rId4"/>
     <sheet name="ДрРоботов" sheetId="5" r:id="rId5"/>
+    <sheet name="ТекПроблем" sheetId="6" r:id="rId6"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="39">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="77" uniqueCount="54">
   <si>
     <t>RL3 - это продолжение RL1</t>
   </si>
@@ -147,15 +157,66 @@
   <si>
     <t>С помощью него можно будет подбирать параметры для PEG30</t>
   </si>
+  <si>
+    <t>PEG31_HYPERION</t>
+  </si>
+  <si>
+    <t>Универсальный сборщик с использование fg</t>
+  </si>
+  <si>
+    <t>Где-то в гиперионе у нас вылетают заявки не в ту сторону, из-за этого он открывает по рынку.</t>
+  </si>
+  <si>
+    <t>В спред часто встает заявка, а под ней пустота в несколько пунктов. Нужно что бы робот их обходил</t>
+  </si>
+  <si>
+    <t>LEG1_CC</t>
+  </si>
+  <si>
+    <t>Адаптация из RL1</t>
+  </si>
+  <si>
+    <t>LEG2_HOTS</t>
+  </si>
+  <si>
+    <t>LEG2_LOGAN</t>
+  </si>
+  <si>
+    <t>WEG4_DOG</t>
+  </si>
+  <si>
+    <t>WT</t>
+  </si>
+  <si>
+    <t>UEG2_GGD</t>
+  </si>
+  <si>
+    <t>UT</t>
+  </si>
+  <si>
+    <t>PEG11_KUSURUKEN</t>
+  </si>
+  <si>
+    <t>SEG3_FORCE</t>
+  </si>
+  <si>
+    <t>PEG20_HOGGER</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -3727,16 +3788,17 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AD38F229-6CC0-4A34-802C-B9D336FEB24E}">
-  <dimension ref="A1:F398"/>
+  <dimension ref="A1:P398"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="21.5703125" customWidth="1"/>
     <col min="3" max="3" width="14" customWidth="1"/>
-    <col min="4" max="4" width="21.5703125" customWidth="1"/>
+    <col min="4" max="4" width="7.28515625" customWidth="1"/>
     <col min="5" max="5" width="44.85546875" customWidth="1"/>
+    <col min="11" max="11" width="14.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="B1" t="s">
         <v>24</v>
       </c>
@@ -3749,8 +3811,23 @@
       <c r="E1" t="s">
         <v>27</v>
       </c>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="L1" t="s">
+        <v>12</v>
+      </c>
+      <c r="M1" t="s">
+        <v>11</v>
+      </c>
+      <c r="N1" t="s">
+        <v>48</v>
+      </c>
+      <c r="O1" t="s">
+        <v>50</v>
+      </c>
+      <c r="P1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="2" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>1</v>
       </c>
@@ -3766,8 +3843,28 @@
       <c r="E2" t="s">
         <v>35</v>
       </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="L2">
+        <f>COUNTIF(D:D,L1)</f>
+        <v>6</v>
+      </c>
+      <c r="M2">
+        <f>COUNTIF(D:D,M1)</f>
+        <v>3</v>
+      </c>
+      <c r="N2">
+        <f>COUNTIF(D:D,N1)</f>
+        <v>1</v>
+      </c>
+      <c r="O2">
+        <f>COUNTIF(D:D,O1)</f>
+        <v>1</v>
+      </c>
+      <c r="P2">
+        <f>COUNTIF(D:D,P1)</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>2</v>
       </c>
@@ -3784,7 +3881,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>3</v>
       </c>
@@ -3804,7 +3901,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>4</v>
       </c>
@@ -3824,57 +3921,165 @@
         <v>38</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>5</v>
       </c>
-    </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="B6" t="s">
+        <v>39</v>
+      </c>
+      <c r="C6" s="3">
+        <v>46246</v>
+      </c>
+      <c r="D6" t="s">
+        <v>12</v>
+      </c>
+      <c r="E6" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="7" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>6</v>
       </c>
-    </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="B7" t="s">
+        <v>43</v>
+      </c>
+      <c r="C7" s="3">
+        <v>46248</v>
+      </c>
+      <c r="D7" t="s">
+        <v>11</v>
+      </c>
+      <c r="E7" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="8" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>7</v>
       </c>
-    </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="B8" t="s">
+        <v>45</v>
+      </c>
+      <c r="C8" s="3">
+        <v>46248</v>
+      </c>
+      <c r="D8" t="s">
+        <v>11</v>
+      </c>
+      <c r="E8" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="9" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>8</v>
       </c>
-    </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="B9" t="s">
+        <v>46</v>
+      </c>
+      <c r="C9" s="3">
+        <v>46248</v>
+      </c>
+      <c r="D9" t="s">
+        <v>11</v>
+      </c>
+      <c r="E9" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="10" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>9</v>
       </c>
-    </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="B10" t="s">
+        <v>47</v>
+      </c>
+      <c r="C10" s="3">
+        <v>46248</v>
+      </c>
+      <c r="D10" t="s">
+        <v>48</v>
+      </c>
+      <c r="E10" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="11" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>10</v>
       </c>
-    </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="B11" t="s">
+        <v>49</v>
+      </c>
+      <c r="C11" s="3">
+        <v>46248</v>
+      </c>
+      <c r="D11" t="s">
+        <v>50</v>
+      </c>
+      <c r="E11" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="12" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A12">
         <v>11</v>
       </c>
-    </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="B12" t="s">
+        <v>51</v>
+      </c>
+      <c r="C12" s="3">
+        <v>46248</v>
+      </c>
+      <c r="D12" t="s">
+        <v>12</v>
+      </c>
+      <c r="E12" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="13" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A13">
         <v>12</v>
       </c>
-    </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="B13" t="s">
+        <v>53</v>
+      </c>
+      <c r="C13" s="3">
+        <v>46248</v>
+      </c>
+      <c r="D13" t="s">
+        <v>12</v>
+      </c>
+      <c r="E13" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="14" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A14">
         <v>13</v>
       </c>
-    </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="B14" t="s">
+        <v>52</v>
+      </c>
+      <c r="C14" s="3">
+        <v>46248</v>
+      </c>
+      <c r="D14" t="s">
+        <v>13</v>
+      </c>
+      <c r="E14" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="15" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A15">
         <v>14</v>
       </c>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A16">
         <v>15</v>
       </c>
@@ -5790,7 +5995,44 @@
       </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D5C6E19E-FDB9-4B9E-B0A7-1D91E81DACEB}">
+  <dimension ref="A2:B5"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A2">
+        <v>1</v>
+      </c>
+      <c r="B2" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A3">
+        <v>2</v>
+      </c>
+      <c r="B3" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A4">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A5">
+        <v>4</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
prepare some group for optima
</commit_message>
<xml_diff>
--- a/__docs/RoadMap.xlsx
+++ b/__docs/RoadMap.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Dev\exchange\RichLaughter3\__docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4634988E-9101-43F7-B9E9-5B99292FA6B7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5CDE63F0-6C44-43E7-8C8A-98D4A91F8708}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1448,9 +1448,6 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
@@ -1465,6 +1462,9 @@
     </xf>
     <xf numFmtId="14" fontId="4" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1799,7 +1799,7 @@
       </c>
     </row>
     <row r="3" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B3" s="7" t="s">
+      <c r="B3" s="12" t="s">
         <v>3</v>
       </c>
       <c r="C3" s="2" t="s">
@@ -1807,13 +1807,13 @@
       </c>
     </row>
     <row r="4" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B4" s="7"/>
+      <c r="B4" s="12"/>
       <c r="C4" s="2" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="5" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B5" s="7" t="s">
+      <c r="B5" s="12" t="s">
         <v>4</v>
       </c>
       <c r="C5" s="2" t="s">
@@ -1821,43 +1821,43 @@
       </c>
     </row>
     <row r="6" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B6" s="7"/>
+      <c r="B6" s="12"/>
       <c r="C6" s="2" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="7" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B7" s="7"/>
+      <c r="B7" s="12"/>
       <c r="C7" s="2" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="8" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B8" s="7"/>
+      <c r="B8" s="12"/>
       <c r="C8" s="2" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="9" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B9" s="7"/>
+      <c r="B9" s="12"/>
       <c r="C9" s="2" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="10" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B10" s="7"/>
+      <c r="B10" s="12"/>
       <c r="C10" s="2" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="11" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B11" s="7"/>
+      <c r="B11" s="12"/>
       <c r="C11" s="2" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="12" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B12" s="7"/>
+      <c r="B12" s="12"/>
       <c r="C12" s="2" t="s">
         <v>17</v>
       </c>
@@ -8261,3636 +8261,3636 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:7" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="B2" s="8" t="s">
+      <c r="B2" s="7" t="s">
         <v>57</v>
       </c>
-      <c r="C2" s="8" t="s">
+      <c r="C2" s="7" t="s">
         <v>58</v>
       </c>
-      <c r="D2" s="8" t="s">
+      <c r="D2" s="7" t="s">
         <v>59</v>
       </c>
-      <c r="E2" s="8" t="s">
+      <c r="E2" s="7" t="s">
         <v>60</v>
       </c>
-      <c r="F2" s="8" t="s">
+      <c r="F2" s="7" t="s">
         <v>61</v>
       </c>
-      <c r="G2" s="8" t="s">
+      <c r="G2" s="7" t="s">
         <v>62</v>
       </c>
     </row>
     <row r="3" spans="2:7" ht="33" x14ac:dyDescent="0.25">
-      <c r="B3" s="9">
+      <c r="B3" s="8">
         <v>1</v>
       </c>
-      <c r="C3" s="10" t="s">
+      <c r="C3" s="9" t="s">
         <v>63</v>
       </c>
-      <c r="D3" s="9" t="s">
+      <c r="D3" s="8" t="s">
         <v>64</v>
       </c>
-      <c r="E3" s="9" t="s">
+      <c r="E3" s="8" t="s">
         <v>65</v>
       </c>
-      <c r="F3" s="11">
+      <c r="F3" s="10">
         <v>46303</v>
       </c>
-      <c r="G3" s="9" t="s">
+      <c r="G3" s="8" t="s">
         <v>66</v>
       </c>
     </row>
     <row r="4" spans="2:7" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="B4" s="9">
+      <c r="B4" s="8">
         <v>2</v>
       </c>
-      <c r="C4" s="10" t="s">
+      <c r="C4" s="9" t="s">
         <v>67</v>
       </c>
-      <c r="D4" s="9" t="s">
+      <c r="D4" s="8" t="s">
         <v>68</v>
       </c>
-      <c r="E4" s="9" t="s">
+      <c r="E4" s="8" t="s">
         <v>69</v>
       </c>
-      <c r="F4" s="12">
+      <c r="F4" s="11">
         <v>40305</v>
       </c>
-      <c r="G4" s="9" t="s">
+      <c r="G4" s="8" t="s">
         <v>70</v>
       </c>
     </row>
     <row r="5" spans="2:7" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="B5" s="9">
+      <c r="B5" s="8">
         <v>3</v>
       </c>
-      <c r="C5" s="10" t="s">
+      <c r="C5" s="9" t="s">
         <v>71</v>
       </c>
-      <c r="D5" s="9" t="s">
+      <c r="D5" s="8" t="s">
         <v>68</v>
       </c>
-      <c r="E5" s="9" t="s">
+      <c r="E5" s="8" t="s">
         <v>72</v>
       </c>
-      <c r="F5" s="12">
+      <c r="F5" s="11">
         <v>40305</v>
       </c>
-      <c r="G5" s="9" t="s">
+      <c r="G5" s="8" t="s">
         <v>70</v>
       </c>
     </row>
     <row r="6" spans="2:7" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="B6" s="9">
+      <c r="B6" s="8">
         <v>4</v>
       </c>
-      <c r="C6" s="10" t="s">
+      <c r="C6" s="9" t="s">
         <v>73</v>
       </c>
-      <c r="D6" s="9" t="s">
+      <c r="D6" s="8" t="s">
         <v>68</v>
       </c>
-      <c r="E6" s="9" t="s">
+      <c r="E6" s="8" t="s">
         <v>74</v>
       </c>
-      <c r="F6" s="12">
+      <c r="F6" s="11">
         <v>40305</v>
       </c>
-      <c r="G6" s="9" t="s">
+      <c r="G6" s="8" t="s">
         <v>70</v>
       </c>
     </row>
     <row r="7" spans="2:7" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="B7" s="9">
+      <c r="B7" s="8">
         <v>5</v>
       </c>
-      <c r="C7" s="10" t="s">
+      <c r="C7" s="9" t="s">
         <v>75</v>
       </c>
-      <c r="D7" s="9" t="s">
+      <c r="D7" s="8" t="s">
         <v>76</v>
       </c>
-      <c r="E7" s="9" t="s">
+      <c r="E7" s="8" t="s">
         <v>77</v>
       </c>
-      <c r="F7" s="12">
+      <c r="F7" s="11">
         <v>40305</v>
       </c>
-      <c r="G7" s="9" t="s">
+      <c r="G7" s="8" t="s">
         <v>70</v>
       </c>
     </row>
     <row r="8" spans="2:7" ht="33" x14ac:dyDescent="0.25">
-      <c r="B8" s="9">
+      <c r="B8" s="8">
         <v>6</v>
       </c>
-      <c r="C8" s="10" t="s">
+      <c r="C8" s="9" t="s">
         <v>78</v>
       </c>
-      <c r="D8" s="9" t="s">
+      <c r="D8" s="8" t="s">
         <v>76</v>
       </c>
-      <c r="E8" s="9" t="s">
+      <c r="E8" s="8" t="s">
         <v>79</v>
       </c>
-      <c r="F8" s="12">
+      <c r="F8" s="11">
         <v>40305</v>
       </c>
-      <c r="G8" s="9" t="s">
+      <c r="G8" s="8" t="s">
         <v>70</v>
       </c>
     </row>
     <row r="9" spans="2:7" ht="33" x14ac:dyDescent="0.25">
-      <c r="B9" s="9">
+      <c r="B9" s="8">
         <v>7</v>
       </c>
-      <c r="C9" s="10" t="s">
+      <c r="C9" s="9" t="s">
         <v>80</v>
       </c>
-      <c r="D9" s="9" t="s">
+      <c r="D9" s="8" t="s">
         <v>76</v>
       </c>
-      <c r="E9" s="9" t="s">
+      <c r="E9" s="8" t="s">
         <v>81</v>
       </c>
-      <c r="F9" s="12">
+      <c r="F9" s="11">
         <v>40305</v>
       </c>
-      <c r="G9" s="9" t="s">
+      <c r="G9" s="8" t="s">
         <v>70</v>
       </c>
     </row>
     <row r="10" spans="2:7" ht="33" x14ac:dyDescent="0.25">
-      <c r="B10" s="9">
+      <c r="B10" s="8">
         <v>8</v>
       </c>
-      <c r="C10" s="10" t="s">
+      <c r="C10" s="9" t="s">
         <v>82</v>
       </c>
-      <c r="D10" s="9" t="s">
+      <c r="D10" s="8" t="s">
         <v>76</v>
       </c>
-      <c r="E10" s="9" t="s">
+      <c r="E10" s="8" t="s">
         <v>83</v>
       </c>
-      <c r="F10" s="12">
+      <c r="F10" s="11">
         <v>40305</v>
       </c>
-      <c r="G10" s="9" t="s">
+      <c r="G10" s="8" t="s">
         <v>70</v>
       </c>
     </row>
     <row r="11" spans="2:7" ht="33" x14ac:dyDescent="0.25">
-      <c r="B11" s="9">
+      <c r="B11" s="8">
         <v>9</v>
       </c>
-      <c r="C11" s="10" t="s">
+      <c r="C11" s="9" t="s">
         <v>84</v>
       </c>
-      <c r="D11" s="9" t="s">
+      <c r="D11" s="8" t="s">
         <v>76</v>
       </c>
-      <c r="E11" s="9" t="s">
+      <c r="E11" s="8" t="s">
         <v>85</v>
       </c>
-      <c r="F11" s="12">
+      <c r="F11" s="11">
         <v>40305</v>
       </c>
-      <c r="G11" s="9" t="s">
+      <c r="G11" s="8" t="s">
         <v>70</v>
       </c>
     </row>
     <row r="12" spans="2:7" ht="33" x14ac:dyDescent="0.25">
-      <c r="B12" s="9">
+      <c r="B12" s="8">
         <v>10</v>
       </c>
-      <c r="C12" s="10" t="s">
+      <c r="C12" s="9" t="s">
         <v>86</v>
       </c>
-      <c r="D12" s="9" t="s">
+      <c r="D12" s="8" t="s">
         <v>76</v>
       </c>
-      <c r="E12" s="9" t="s">
+      <c r="E12" s="8" t="s">
         <v>87</v>
       </c>
-      <c r="F12" s="12">
+      <c r="F12" s="11">
         <v>40305</v>
       </c>
-      <c r="G12" s="9" t="s">
+      <c r="G12" s="8" t="s">
         <v>70</v>
       </c>
     </row>
     <row r="13" spans="2:7" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="B13" s="9">
+      <c r="B13" s="8">
         <v>11</v>
       </c>
-      <c r="C13" s="10" t="s">
+      <c r="C13" s="9" t="s">
         <v>88</v>
       </c>
-      <c r="D13" s="9" t="s">
+      <c r="D13" s="8" t="s">
         <v>89</v>
       </c>
-      <c r="E13" s="9" t="s">
+      <c r="E13" s="8" t="s">
         <v>90</v>
       </c>
-      <c r="F13" s="12">
+      <c r="F13" s="11">
         <v>40305</v>
       </c>
-      <c r="G13" s="9" t="s">
+      <c r="G13" s="8" t="s">
         <v>70</v>
       </c>
     </row>
     <row r="14" spans="2:7" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="B14" s="9">
+      <c r="B14" s="8">
         <v>12</v>
       </c>
-      <c r="C14" s="10" t="s">
+      <c r="C14" s="9" t="s">
         <v>91</v>
       </c>
-      <c r="D14" s="9" t="s">
+      <c r="D14" s="8" t="s">
         <v>64</v>
       </c>
-      <c r="E14" s="9" t="s">
+      <c r="E14" s="8" t="s">
         <v>92</v>
       </c>
-      <c r="F14" s="12">
+      <c r="F14" s="11">
         <v>40305</v>
       </c>
-      <c r="G14" s="9" t="s">
+      <c r="G14" s="8" t="s">
         <v>70</v>
       </c>
     </row>
     <row r="15" spans="2:7" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="B15" s="9">
+      <c r="B15" s="8">
         <v>13</v>
       </c>
-      <c r="C15" s="10" t="s">
+      <c r="C15" s="9" t="s">
         <v>93</v>
       </c>
-      <c r="D15" s="9" t="s">
+      <c r="D15" s="8" t="s">
         <v>94</v>
       </c>
-      <c r="E15" s="9" t="s">
+      <c r="E15" s="8" t="s">
         <v>95</v>
       </c>
-      <c r="F15" s="12">
+      <c r="F15" s="11">
         <v>40305</v>
       </c>
-      <c r="G15" s="9" t="s">
+      <c r="G15" s="8" t="s">
         <v>70</v>
       </c>
     </row>
     <row r="16" spans="2:7" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="B16" s="9">
+      <c r="B16" s="8">
         <v>14</v>
       </c>
-      <c r="C16" s="10" t="s">
+      <c r="C16" s="9" t="s">
         <v>96</v>
       </c>
-      <c r="D16" s="9" t="s">
+      <c r="D16" s="8" t="s">
         <v>68</v>
       </c>
-      <c r="E16" s="9" t="s">
+      <c r="E16" s="8" t="s">
         <v>97</v>
       </c>
-      <c r="F16" s="11">
+      <c r="F16" s="10">
         <v>46302</v>
       </c>
-      <c r="G16" s="9" t="s">
+      <c r="G16" s="8" t="s">
         <v>70</v>
       </c>
     </row>
     <row r="17" spans="2:7" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="B17" s="9">
+      <c r="B17" s="8">
         <v>15</v>
       </c>
-      <c r="C17" s="10" t="s">
+      <c r="C17" s="9" t="s">
         <v>98</v>
       </c>
-      <c r="D17" s="9" t="s">
+      <c r="D17" s="8" t="s">
         <v>68</v>
       </c>
-      <c r="E17" s="9" t="s">
+      <c r="E17" s="8" t="s">
         <v>99</v>
       </c>
-      <c r="F17" s="11">
+      <c r="F17" s="10">
         <v>46302</v>
       </c>
-      <c r="G17" s="9" t="s">
+      <c r="G17" s="8" t="s">
         <v>70</v>
       </c>
     </row>
     <row r="18" spans="2:7" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="B18" s="9">
+      <c r="B18" s="8">
         <v>16</v>
       </c>
-      <c r="C18" s="10" t="s">
+      <c r="C18" s="9" t="s">
         <v>100</v>
       </c>
-      <c r="D18" s="9" t="s">
+      <c r="D18" s="8" t="s">
         <v>68</v>
       </c>
-      <c r="E18" s="9" t="s">
+      <c r="E18" s="8" t="s">
         <v>101</v>
       </c>
-      <c r="F18" s="11">
+      <c r="F18" s="10">
         <v>46302</v>
       </c>
-      <c r="G18" s="9" t="s">
+      <c r="G18" s="8" t="s">
         <v>70</v>
       </c>
     </row>
     <row r="19" spans="2:7" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="B19" s="9">
+      <c r="B19" s="8">
         <v>17</v>
       </c>
-      <c r="C19" s="10" t="s">
+      <c r="C19" s="9" t="s">
         <v>102</v>
       </c>
-      <c r="D19" s="9" t="s">
+      <c r="D19" s="8" t="s">
         <v>68</v>
       </c>
-      <c r="E19" s="9" t="s">
+      <c r="E19" s="8" t="s">
         <v>103</v>
       </c>
-      <c r="F19" s="11">
+      <c r="F19" s="10">
         <v>46302</v>
       </c>
-      <c r="G19" s="9" t="s">
+      <c r="G19" s="8" t="s">
         <v>70</v>
       </c>
     </row>
     <row r="20" spans="2:7" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="B20" s="9">
+      <c r="B20" s="8">
         <v>18</v>
       </c>
-      <c r="C20" s="10" t="s">
+      <c r="C20" s="9" t="s">
         <v>104</v>
       </c>
-      <c r="D20" s="9" t="s">
+      <c r="D20" s="8" t="s">
         <v>68</v>
       </c>
-      <c r="E20" s="9" t="s">
+      <c r="E20" s="8" t="s">
         <v>105</v>
       </c>
-      <c r="F20" s="11">
+      <c r="F20" s="10">
         <v>46302</v>
       </c>
-      <c r="G20" s="9" t="s">
+      <c r="G20" s="8" t="s">
         <v>70</v>
       </c>
     </row>
     <row r="21" spans="2:7" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="B21" s="9">
+      <c r="B21" s="8">
         <v>19</v>
       </c>
-      <c r="C21" s="10" t="s">
+      <c r="C21" s="9" t="s">
         <v>106</v>
       </c>
-      <c r="D21" s="9" t="s">
+      <c r="D21" s="8" t="s">
         <v>68</v>
       </c>
-      <c r="E21" s="9" t="s">
+      <c r="E21" s="8" t="s">
         <v>107</v>
       </c>
-      <c r="F21" s="11">
+      <c r="F21" s="10">
         <v>46302</v>
       </c>
-      <c r="G21" s="9" t="s">
+      <c r="G21" s="8" t="s">
         <v>70</v>
       </c>
     </row>
     <row r="22" spans="2:7" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="B22" s="9">
+      <c r="B22" s="8">
         <v>20</v>
       </c>
-      <c r="C22" s="10" t="s">
+      <c r="C22" s="9" t="s">
         <v>108</v>
       </c>
-      <c r="D22" s="9" t="s">
+      <c r="D22" s="8" t="s">
         <v>76</v>
       </c>
-      <c r="E22" s="9" t="s">
+      <c r="E22" s="8" t="s">
         <v>109</v>
       </c>
-      <c r="F22" s="11">
+      <c r="F22" s="10">
         <v>46302</v>
       </c>
-      <c r="G22" s="9" t="s">
+      <c r="G22" s="8" t="s">
         <v>70</v>
       </c>
     </row>
     <row r="23" spans="2:7" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="B23" s="9">
+      <c r="B23" s="8">
         <v>21</v>
       </c>
-      <c r="C23" s="10" t="s">
+      <c r="C23" s="9" t="s">
         <v>110</v>
       </c>
-      <c r="D23" s="9" t="s">
+      <c r="D23" s="8" t="s">
         <v>76</v>
       </c>
-      <c r="E23" s="9" t="s">
+      <c r="E23" s="8" t="s">
         <v>111</v>
       </c>
-      <c r="F23" s="11">
+      <c r="F23" s="10">
         <v>46302</v>
       </c>
-      <c r="G23" s="9" t="s">
+      <c r="G23" s="8" t="s">
         <v>70</v>
       </c>
     </row>
     <row r="24" spans="2:7" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="B24" s="9">
+      <c r="B24" s="8">
         <v>22</v>
       </c>
-      <c r="C24" s="10" t="s">
+      <c r="C24" s="9" t="s">
         <v>112</v>
       </c>
-      <c r="D24" s="9" t="s">
+      <c r="D24" s="8" t="s">
         <v>76</v>
       </c>
-      <c r="E24" s="9" t="s">
+      <c r="E24" s="8" t="s">
         <v>113</v>
       </c>
-      <c r="F24" s="12">
+      <c r="F24" s="11">
         <v>40305</v>
       </c>
-      <c r="G24" s="9" t="s">
+      <c r="G24" s="8" t="s">
         <v>70</v>
       </c>
     </row>
     <row r="25" spans="2:7" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="B25" s="9">
+      <c r="B25" s="8">
         <v>23</v>
       </c>
-      <c r="C25" s="10" t="s">
+      <c r="C25" s="9" t="s">
         <v>114</v>
       </c>
-      <c r="D25" s="9" t="s">
+      <c r="D25" s="8" t="s">
         <v>76</v>
       </c>
-      <c r="E25" s="9" t="s">
+      <c r="E25" s="8" t="s">
         <v>115</v>
       </c>
-      <c r="F25" s="12">
+      <c r="F25" s="11">
         <v>40305</v>
       </c>
-      <c r="G25" s="9" t="s">
+      <c r="G25" s="8" t="s">
         <v>70</v>
       </c>
     </row>
     <row r="26" spans="2:7" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="B26" s="9">
+      <c r="B26" s="8">
         <v>24</v>
       </c>
-      <c r="C26" s="10" t="s">
+      <c r="C26" s="9" t="s">
         <v>116</v>
       </c>
-      <c r="D26" s="9" t="s">
+      <c r="D26" s="8" t="s">
         <v>76</v>
       </c>
-      <c r="E26" s="9" t="s">
+      <c r="E26" s="8" t="s">
         <v>117</v>
       </c>
-      <c r="F26" s="12">
+      <c r="F26" s="11">
         <v>40304</v>
       </c>
-      <c r="G26" s="9" t="s">
+      <c r="G26" s="8" t="s">
         <v>118</v>
       </c>
     </row>
     <row r="27" spans="2:7" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="B27" s="9">
+      <c r="B27" s="8">
         <v>25</v>
       </c>
-      <c r="C27" s="10" t="s">
+      <c r="C27" s="9" t="s">
         <v>119</v>
       </c>
-      <c r="D27" s="9" t="s">
+      <c r="D27" s="8" t="s">
         <v>76</v>
       </c>
-      <c r="E27" s="9" t="s">
+      <c r="E27" s="8" t="s">
         <v>120</v>
       </c>
-      <c r="F27" s="12">
+      <c r="F27" s="11">
         <v>40304</v>
       </c>
-      <c r="G27" s="9" t="s">
+      <c r="G27" s="8" t="s">
         <v>118</v>
       </c>
     </row>
     <row r="28" spans="2:7" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="B28" s="9">
+      <c r="B28" s="8">
         <v>26</v>
       </c>
-      <c r="C28" s="10" t="s">
+      <c r="C28" s="9" t="s">
         <v>121</v>
       </c>
-      <c r="D28" s="9" t="s">
+      <c r="D28" s="8" t="s">
         <v>76</v>
       </c>
-      <c r="E28" s="9" t="s">
+      <c r="E28" s="8" t="s">
         <v>122</v>
       </c>
-      <c r="F28" s="11">
+      <c r="F28" s="10">
         <v>46302</v>
       </c>
-      <c r="G28" s="9" t="s">
+      <c r="G28" s="8" t="s">
         <v>70</v>
       </c>
     </row>
     <row r="29" spans="2:7" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="B29" s="9">
+      <c r="B29" s="8">
         <v>27</v>
       </c>
-      <c r="C29" s="10" t="s">
+      <c r="C29" s="9" t="s">
         <v>123</v>
       </c>
-      <c r="D29" s="9" t="s">
+      <c r="D29" s="8" t="s">
         <v>76</v>
       </c>
-      <c r="E29" s="9" t="s">
+      <c r="E29" s="8" t="s">
         <v>124</v>
       </c>
-      <c r="F29" s="11">
+      <c r="F29" s="10">
         <v>46302</v>
       </c>
-      <c r="G29" s="9" t="s">
+      <c r="G29" s="8" t="s">
         <v>70</v>
       </c>
     </row>
     <row r="30" spans="2:7" ht="33" x14ac:dyDescent="0.25">
-      <c r="B30" s="9">
+      <c r="B30" s="8">
         <v>28</v>
       </c>
-      <c r="C30" s="10" t="s">
+      <c r="C30" s="9" t="s">
         <v>125</v>
       </c>
-      <c r="D30" s="9" t="s">
+      <c r="D30" s="8" t="s">
         <v>76</v>
       </c>
-      <c r="E30" s="9" t="s">
+      <c r="E30" s="8" t="s">
         <v>126</v>
       </c>
-      <c r="F30" s="11">
+      <c r="F30" s="10">
         <v>46302</v>
       </c>
-      <c r="G30" s="9" t="s">
+      <c r="G30" s="8" t="s">
         <v>70</v>
       </c>
     </row>
     <row r="31" spans="2:7" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="B31" s="9">
+      <c r="B31" s="8">
         <v>29</v>
       </c>
-      <c r="C31" s="10" t="s">
+      <c r="C31" s="9" t="s">
         <v>127</v>
       </c>
-      <c r="D31" s="9" t="s">
+      <c r="D31" s="8" t="s">
         <v>76</v>
       </c>
-      <c r="E31" s="9" t="s">
+      <c r="E31" s="8" t="s">
         <v>128</v>
       </c>
-      <c r="F31" s="11">
+      <c r="F31" s="10">
         <v>46302</v>
       </c>
-      <c r="G31" s="9" t="s">
+      <c r="G31" s="8" t="s">
         <v>70</v>
       </c>
     </row>
     <row r="32" spans="2:7" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="B32" s="9">
+      <c r="B32" s="8">
         <v>30</v>
       </c>
-      <c r="C32" s="10" t="s">
+      <c r="C32" s="9" t="s">
         <v>129</v>
       </c>
-      <c r="D32" s="9" t="s">
+      <c r="D32" s="8" t="s">
         <v>76</v>
       </c>
-      <c r="E32" s="9" t="s">
+      <c r="E32" s="8" t="s">
         <v>130</v>
       </c>
-      <c r="F32" s="11">
+      <c r="F32" s="10">
         <v>46302</v>
       </c>
-      <c r="G32" s="9" t="s">
+      <c r="G32" s="8" t="s">
         <v>70</v>
       </c>
     </row>
     <row r="33" spans="2:7" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="B33" s="9">
+      <c r="B33" s="8">
         <v>31</v>
       </c>
-      <c r="C33" s="10" t="s">
+      <c r="C33" s="9" t="s">
         <v>131</v>
       </c>
-      <c r="D33" s="9" t="s">
+      <c r="D33" s="8" t="s">
         <v>76</v>
       </c>
-      <c r="E33" s="9" t="s">
+      <c r="E33" s="8" t="s">
         <v>132</v>
       </c>
-      <c r="F33" s="11">
+      <c r="F33" s="10">
         <v>46302</v>
       </c>
-      <c r="G33" s="9" t="s">
+      <c r="G33" s="8" t="s">
         <v>70</v>
       </c>
     </row>
     <row r="34" spans="2:7" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="B34" s="9">
+      <c r="B34" s="8">
         <v>32</v>
       </c>
-      <c r="C34" s="10" t="s">
+      <c r="C34" s="9" t="s">
         <v>133</v>
       </c>
-      <c r="D34" s="9" t="s">
+      <c r="D34" s="8" t="s">
         <v>76</v>
       </c>
-      <c r="E34" s="9" t="s">
+      <c r="E34" s="8" t="s">
         <v>134</v>
       </c>
-      <c r="F34" s="11">
+      <c r="F34" s="10">
         <v>46302</v>
       </c>
-      <c r="G34" s="9" t="s">
+      <c r="G34" s="8" t="s">
         <v>70</v>
       </c>
     </row>
     <row r="35" spans="2:7" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="B35" s="9">
+      <c r="B35" s="8">
         <v>33</v>
       </c>
-      <c r="C35" s="10" t="s">
+      <c r="C35" s="9" t="s">
         <v>135</v>
       </c>
-      <c r="D35" s="9" t="s">
+      <c r="D35" s="8" t="s">
         <v>76</v>
       </c>
-      <c r="E35" s="9" t="s">
+      <c r="E35" s="8" t="s">
         <v>136</v>
       </c>
-      <c r="F35" s="11">
+      <c r="F35" s="10">
         <v>46302</v>
       </c>
-      <c r="G35" s="9" t="s">
+      <c r="G35" s="8" t="s">
         <v>70</v>
       </c>
     </row>
     <row r="36" spans="2:7" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="B36" s="9">
+      <c r="B36" s="8">
         <v>34</v>
       </c>
-      <c r="C36" s="10" t="s">
+      <c r="C36" s="9" t="s">
         <v>137</v>
       </c>
-      <c r="D36" s="9" t="s">
+      <c r="D36" s="8" t="s">
         <v>76</v>
       </c>
-      <c r="E36" s="9" t="s">
+      <c r="E36" s="8" t="s">
         <v>138</v>
       </c>
-      <c r="F36" s="11">
+      <c r="F36" s="10">
         <v>46302</v>
       </c>
-      <c r="G36" s="9" t="s">
+      <c r="G36" s="8" t="s">
         <v>70</v>
       </c>
     </row>
     <row r="37" spans="2:7" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="B37" s="9">
+      <c r="B37" s="8">
         <v>35</v>
       </c>
-      <c r="C37" s="10" t="s">
+      <c r="C37" s="9" t="s">
         <v>139</v>
       </c>
-      <c r="D37" s="9" t="s">
+      <c r="D37" s="8" t="s">
         <v>76</v>
       </c>
-      <c r="E37" s="9" t="s">
+      <c r="E37" s="8" t="s">
         <v>140</v>
       </c>
-      <c r="F37" s="11">
+      <c r="F37" s="10">
         <v>46302</v>
       </c>
-      <c r="G37" s="9" t="s">
+      <c r="G37" s="8" t="s">
         <v>70</v>
       </c>
     </row>
     <row r="38" spans="2:7" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="B38" s="9">
+      <c r="B38" s="8">
         <v>36</v>
       </c>
-      <c r="C38" s="10" t="s">
+      <c r="C38" s="9" t="s">
         <v>141</v>
       </c>
-      <c r="D38" s="9" t="s">
+      <c r="D38" s="8" t="s">
         <v>76</v>
       </c>
-      <c r="E38" s="9" t="s">
+      <c r="E38" s="8" t="s">
         <v>142</v>
       </c>
-      <c r="F38" s="11">
+      <c r="F38" s="10">
         <v>46302</v>
       </c>
-      <c r="G38" s="9" t="s">
+      <c r="G38" s="8" t="s">
         <v>70</v>
       </c>
     </row>
     <row r="39" spans="2:7" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="B39" s="9">
+      <c r="B39" s="8">
         <v>37</v>
       </c>
-      <c r="C39" s="10" t="s">
+      <c r="C39" s="9" t="s">
         <v>143</v>
       </c>
-      <c r="D39" s="9" t="s">
+      <c r="D39" s="8" t="s">
         <v>76</v>
       </c>
-      <c r="E39" s="9" t="s">
+      <c r="E39" s="8" t="s">
         <v>144</v>
       </c>
-      <c r="F39" s="11">
+      <c r="F39" s="10">
         <v>46302</v>
       </c>
-      <c r="G39" s="9" t="s">
+      <c r="G39" s="8" t="s">
         <v>70</v>
       </c>
     </row>
     <row r="40" spans="2:7" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="B40" s="9">
+      <c r="B40" s="8">
         <v>38</v>
       </c>
-      <c r="C40" s="10" t="s">
+      <c r="C40" s="9" t="s">
         <v>145</v>
       </c>
-      <c r="D40" s="9" t="s">
+      <c r="D40" s="8" t="s">
         <v>76</v>
       </c>
-      <c r="E40" s="9" t="s">
+      <c r="E40" s="8" t="s">
         <v>144</v>
       </c>
-      <c r="F40" s="11">
+      <c r="F40" s="10">
         <v>46302</v>
       </c>
-      <c r="G40" s="9" t="s">
+      <c r="G40" s="8" t="s">
         <v>70</v>
       </c>
     </row>
     <row r="41" spans="2:7" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="B41" s="9">
+      <c r="B41" s="8">
         <v>39</v>
       </c>
-      <c r="C41" s="10" t="s">
+      <c r="C41" s="9" t="s">
         <v>146</v>
       </c>
-      <c r="D41" s="9" t="s">
+      <c r="D41" s="8" t="s">
         <v>76</v>
       </c>
-      <c r="E41" s="9" t="s">
+      <c r="E41" s="8" t="s">
         <v>147</v>
       </c>
-      <c r="F41" s="11">
+      <c r="F41" s="10">
         <v>46302</v>
       </c>
-      <c r="G41" s="9" t="s">
+      <c r="G41" s="8" t="s">
         <v>70</v>
       </c>
     </row>
     <row r="42" spans="2:7" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="B42" s="9">
+      <c r="B42" s="8">
         <v>40</v>
       </c>
-      <c r="C42" s="10" t="s">
+      <c r="C42" s="9" t="s">
         <v>148</v>
       </c>
-      <c r="D42" s="9" t="s">
+      <c r="D42" s="8" t="s">
         <v>76</v>
       </c>
-      <c r="E42" s="9" t="s">
+      <c r="E42" s="8" t="s">
         <v>149</v>
       </c>
-      <c r="F42" s="11">
+      <c r="F42" s="10">
         <v>46302</v>
       </c>
-      <c r="G42" s="9" t="s">
+      <c r="G42" s="8" t="s">
         <v>70</v>
       </c>
     </row>
     <row r="43" spans="2:7" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="B43" s="9">
+      <c r="B43" s="8">
         <v>41</v>
       </c>
-      <c r="C43" s="10" t="s">
+      <c r="C43" s="9" t="s">
         <v>150</v>
       </c>
-      <c r="D43" s="9" t="s">
+      <c r="D43" s="8" t="s">
         <v>76</v>
       </c>
-      <c r="E43" s="9" t="s">
+      <c r="E43" s="8" t="s">
         <v>151</v>
       </c>
-      <c r="F43" s="11">
+      <c r="F43" s="10">
         <v>46302</v>
       </c>
-      <c r="G43" s="9" t="s">
+      <c r="G43" s="8" t="s">
         <v>70</v>
       </c>
     </row>
     <row r="44" spans="2:7" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="B44" s="9">
+      <c r="B44" s="8">
         <v>42</v>
       </c>
-      <c r="C44" s="10" t="s">
+      <c r="C44" s="9" t="s">
         <v>152</v>
       </c>
-      <c r="D44" s="9" t="s">
+      <c r="D44" s="8" t="s">
         <v>76</v>
       </c>
-      <c r="E44" s="9" t="s">
+      <c r="E44" s="8" t="s">
         <v>153</v>
       </c>
-      <c r="F44" s="11">
+      <c r="F44" s="10">
         <v>46302</v>
       </c>
-      <c r="G44" s="9" t="s">
+      <c r="G44" s="8" t="s">
         <v>70</v>
       </c>
     </row>
     <row r="45" spans="2:7" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="B45" s="9">
+      <c r="B45" s="8">
         <v>43</v>
       </c>
-      <c r="C45" s="10" t="s">
+      <c r="C45" s="9" t="s">
         <v>154</v>
       </c>
-      <c r="D45" s="9" t="s">
+      <c r="D45" s="8" t="s">
         <v>76</v>
       </c>
-      <c r="E45" s="9" t="s">
+      <c r="E45" s="8" t="s">
         <v>155</v>
       </c>
-      <c r="F45" s="11">
+      <c r="F45" s="10">
         <v>46302</v>
       </c>
-      <c r="G45" s="9" t="s">
+      <c r="G45" s="8" t="s">
         <v>70</v>
       </c>
     </row>
     <row r="46" spans="2:7" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="B46" s="9">
+      <c r="B46" s="8">
         <v>44</v>
       </c>
-      <c r="C46" s="10" t="s">
+      <c r="C46" s="9" t="s">
         <v>156</v>
       </c>
-      <c r="D46" s="9" t="s">
+      <c r="D46" s="8" t="s">
         <v>76</v>
       </c>
-      <c r="E46" s="9" t="s">
+      <c r="E46" s="8" t="s">
         <v>157</v>
       </c>
-      <c r="F46" s="11">
+      <c r="F46" s="10">
         <v>46302</v>
       </c>
-      <c r="G46" s="9" t="s">
+      <c r="G46" s="8" t="s">
         <v>70</v>
       </c>
     </row>
     <row r="47" spans="2:7" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="B47" s="9">
+      <c r="B47" s="8">
         <v>45</v>
       </c>
-      <c r="C47" s="10" t="s">
+      <c r="C47" s="9" t="s">
         <v>158</v>
       </c>
-      <c r="D47" s="9" t="s">
+      <c r="D47" s="8" t="s">
         <v>76</v>
       </c>
-      <c r="E47" s="9" t="s">
+      <c r="E47" s="8" t="s">
         <v>159</v>
       </c>
-      <c r="F47" s="12">
+      <c r="F47" s="11">
         <v>40305</v>
       </c>
-      <c r="G47" s="9" t="s">
+      <c r="G47" s="8" t="s">
         <v>70</v>
       </c>
     </row>
     <row r="48" spans="2:7" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="B48" s="9">
+      <c r="B48" s="8">
         <v>46</v>
       </c>
-      <c r="C48" s="10" t="s">
+      <c r="C48" s="9" t="s">
         <v>160</v>
       </c>
-      <c r="D48" s="9" t="s">
+      <c r="D48" s="8" t="s">
         <v>76</v>
       </c>
-      <c r="E48" s="9" t="s">
+      <c r="E48" s="8" t="s">
         <v>161</v>
       </c>
-      <c r="F48" s="12">
+      <c r="F48" s="11">
         <v>40305</v>
       </c>
-      <c r="G48" s="9" t="s">
+      <c r="G48" s="8" t="s">
         <v>70</v>
       </c>
     </row>
     <row r="49" spans="2:7" ht="33" x14ac:dyDescent="0.25">
-      <c r="B49" s="9">
+      <c r="B49" s="8">
         <v>47</v>
       </c>
-      <c r="C49" s="10" t="s">
+      <c r="C49" s="9" t="s">
         <v>162</v>
       </c>
-      <c r="D49" s="9" t="s">
+      <c r="D49" s="8" t="s">
         <v>76</v>
       </c>
-      <c r="E49" s="9" t="s">
+      <c r="E49" s="8" t="s">
         <v>163</v>
       </c>
-      <c r="F49" s="12">
+      <c r="F49" s="11">
         <v>40305</v>
       </c>
-      <c r="G49" s="9" t="s">
+      <c r="G49" s="8" t="s">
         <v>70</v>
       </c>
     </row>
     <row r="50" spans="2:7" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="B50" s="9">
+      <c r="B50" s="8">
         <v>48</v>
       </c>
-      <c r="C50" s="10" t="s">
+      <c r="C50" s="9" t="s">
         <v>164</v>
       </c>
-      <c r="D50" s="9" t="s">
+      <c r="D50" s="8" t="s">
         <v>76</v>
       </c>
-      <c r="E50" s="9" t="s">
+      <c r="E50" s="8" t="s">
         <v>165</v>
       </c>
-      <c r="F50" s="12">
+      <c r="F50" s="11">
         <v>40305</v>
       </c>
-      <c r="G50" s="9" t="s">
+      <c r="G50" s="8" t="s">
         <v>70</v>
       </c>
     </row>
     <row r="51" spans="2:7" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="B51" s="9">
+      <c r="B51" s="8">
         <v>49</v>
       </c>
-      <c r="C51" s="10" t="s">
+      <c r="C51" s="9" t="s">
         <v>166</v>
       </c>
-      <c r="D51" s="9" t="s">
+      <c r="D51" s="8" t="s">
         <v>76</v>
       </c>
-      <c r="E51" s="9" t="s">
+      <c r="E51" s="8" t="s">
         <v>167</v>
       </c>
-      <c r="F51" s="11">
+      <c r="F51" s="10">
         <v>46302</v>
       </c>
-      <c r="G51" s="9" t="s">
+      <c r="G51" s="8" t="s">
         <v>70</v>
       </c>
     </row>
     <row r="52" spans="2:7" ht="33" x14ac:dyDescent="0.25">
-      <c r="B52" s="9">
+      <c r="B52" s="8">
         <v>50</v>
       </c>
-      <c r="C52" s="10" t="s">
+      <c r="C52" s="9" t="s">
         <v>168</v>
       </c>
-      <c r="D52" s="9" t="s">
+      <c r="D52" s="8" t="s">
         <v>76</v>
       </c>
-      <c r="E52" s="9" t="s">
+      <c r="E52" s="8" t="s">
         <v>169</v>
       </c>
-      <c r="F52" s="12">
+      <c r="F52" s="11">
         <v>40305</v>
       </c>
-      <c r="G52" s="9" t="s">
+      <c r="G52" s="8" t="s">
         <v>70</v>
       </c>
     </row>
     <row r="53" spans="2:7" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="B53" s="9">
+      <c r="B53" s="8">
         <v>51</v>
       </c>
-      <c r="C53" s="10" t="s">
+      <c r="C53" s="9" t="s">
         <v>170</v>
       </c>
-      <c r="D53" s="9" t="s">
+      <c r="D53" s="8" t="s">
         <v>76</v>
       </c>
-      <c r="E53" s="9" t="s">
+      <c r="E53" s="8" t="s">
         <v>171</v>
       </c>
-      <c r="F53" s="12">
+      <c r="F53" s="11">
         <v>40305</v>
       </c>
-      <c r="G53" s="9" t="s">
+      <c r="G53" s="8" t="s">
         <v>70</v>
       </c>
     </row>
     <row r="54" spans="2:7" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="B54" s="9">
+      <c r="B54" s="8">
         <v>52</v>
       </c>
-      <c r="C54" s="10" t="s">
+      <c r="C54" s="9" t="s">
         <v>172</v>
       </c>
-      <c r="D54" s="9" t="s">
+      <c r="D54" s="8" t="s">
         <v>76</v>
       </c>
-      <c r="E54" s="9" t="s">
+      <c r="E54" s="8" t="s">
         <v>173</v>
       </c>
-      <c r="F54" s="12">
+      <c r="F54" s="11">
         <v>40305</v>
       </c>
-      <c r="G54" s="9" t="s">
+      <c r="G54" s="8" t="s">
         <v>70</v>
       </c>
     </row>
     <row r="55" spans="2:7" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="B55" s="9">
+      <c r="B55" s="8">
         <v>53</v>
       </c>
-      <c r="C55" s="10" t="s">
+      <c r="C55" s="9" t="s">
         <v>174</v>
       </c>
-      <c r="D55" s="9" t="s">
+      <c r="D55" s="8" t="s">
         <v>76</v>
       </c>
-      <c r="E55" s="9" t="s">
+      <c r="E55" s="8" t="s">
         <v>173</v>
       </c>
-      <c r="F55" s="11">
+      <c r="F55" s="10">
         <v>46302</v>
       </c>
-      <c r="G55" s="9" t="s">
+      <c r="G55" s="8" t="s">
         <v>70</v>
       </c>
     </row>
     <row r="56" spans="2:7" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="B56" s="9">
+      <c r="B56" s="8">
         <v>54</v>
       </c>
-      <c r="C56" s="10" t="s">
+      <c r="C56" s="9" t="s">
         <v>175</v>
       </c>
-      <c r="D56" s="9" t="s">
+      <c r="D56" s="8" t="s">
         <v>76</v>
       </c>
-      <c r="E56" s="9" t="s">
+      <c r="E56" s="8" t="s">
         <v>176</v>
       </c>
-      <c r="F56" s="12">
+      <c r="F56" s="11">
         <v>40305</v>
       </c>
-      <c r="G56" s="9" t="s">
+      <c r="G56" s="8" t="s">
         <v>70</v>
       </c>
     </row>
     <row r="57" spans="2:7" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="B57" s="9">
+      <c r="B57" s="8">
         <v>55</v>
       </c>
-      <c r="C57" s="10" t="s">
+      <c r="C57" s="9" t="s">
         <v>177</v>
       </c>
-      <c r="D57" s="9" t="s">
+      <c r="D57" s="8" t="s">
         <v>76</v>
       </c>
-      <c r="E57" s="9" t="s">
+      <c r="E57" s="8" t="s">
         <v>178</v>
       </c>
-      <c r="F57" s="12">
+      <c r="F57" s="11">
         <v>40305</v>
       </c>
-      <c r="G57" s="9" t="s">
+      <c r="G57" s="8" t="s">
         <v>70</v>
       </c>
     </row>
     <row r="58" spans="2:7" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="B58" s="9">
+      <c r="B58" s="8">
         <v>56</v>
       </c>
-      <c r="C58" s="10" t="s">
+      <c r="C58" s="9" t="s">
         <v>179</v>
       </c>
-      <c r="D58" s="9" t="s">
+      <c r="D58" s="8" t="s">
         <v>89</v>
       </c>
-      <c r="E58" s="9" t="s">
+      <c r="E58" s="8" t="s">
         <v>180</v>
       </c>
-      <c r="F58" s="11">
+      <c r="F58" s="10">
         <v>46302</v>
       </c>
-      <c r="G58" s="9" t="s">
+      <c r="G58" s="8" t="s">
         <v>70</v>
       </c>
     </row>
     <row r="59" spans="2:7" ht="33" x14ac:dyDescent="0.25">
-      <c r="B59" s="9">
+      <c r="B59" s="8">
         <v>57</v>
       </c>
-      <c r="C59" s="10" t="s">
+      <c r="C59" s="9" t="s">
         <v>181</v>
       </c>
-      <c r="D59" s="9" t="s">
+      <c r="D59" s="8" t="s">
         <v>89</v>
       </c>
-      <c r="E59" s="9" t="s">
+      <c r="E59" s="8" t="s">
         <v>182</v>
       </c>
-      <c r="F59" s="11">
+      <c r="F59" s="10">
         <v>46302</v>
       </c>
-      <c r="G59" s="9" t="s">
+      <c r="G59" s="8" t="s">
         <v>70</v>
       </c>
     </row>
     <row r="60" spans="2:7" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="B60" s="9">
+      <c r="B60" s="8">
         <v>58</v>
       </c>
-      <c r="C60" s="10" t="s">
+      <c r="C60" s="9" t="s">
         <v>183</v>
       </c>
-      <c r="D60" s="9" t="s">
+      <c r="D60" s="8" t="s">
         <v>89</v>
       </c>
-      <c r="E60" s="9" t="s">
+      <c r="E60" s="8" t="s">
         <v>184</v>
       </c>
-      <c r="F60" s="12">
+      <c r="F60" s="11">
         <v>40305</v>
       </c>
-      <c r="G60" s="9" t="s">
+      <c r="G60" s="8" t="s">
         <v>70</v>
       </c>
     </row>
     <row r="61" spans="2:7" ht="33" x14ac:dyDescent="0.25">
-      <c r="B61" s="9">
+      <c r="B61" s="8">
         <v>59</v>
       </c>
-      <c r="C61" s="10" t="s">
+      <c r="C61" s="9" t="s">
         <v>185</v>
       </c>
-      <c r="D61" s="9" t="s">
+      <c r="D61" s="8" t="s">
         <v>89</v>
       </c>
-      <c r="E61" s="9" t="s">
+      <c r="E61" s="8" t="s">
         <v>186</v>
       </c>
-      <c r="F61" s="12">
+      <c r="F61" s="11">
         <v>40305</v>
       </c>
-      <c r="G61" s="9" t="s">
+      <c r="G61" s="8" t="s">
         <v>70</v>
       </c>
     </row>
     <row r="62" spans="2:7" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="B62" s="9">
+      <c r="B62" s="8">
         <v>60</v>
       </c>
-      <c r="C62" s="10" t="s">
+      <c r="C62" s="9" t="s">
         <v>187</v>
       </c>
-      <c r="D62" s="9" t="s">
+      <c r="D62" s="8" t="s">
         <v>188</v>
       </c>
-      <c r="E62" s="9" t="s">
+      <c r="E62" s="8" t="s">
         <v>189</v>
       </c>
-      <c r="F62" s="12">
+      <c r="F62" s="11">
         <v>40305</v>
       </c>
-      <c r="G62" s="9" t="s">
+      <c r="G62" s="8" t="s">
         <v>70</v>
       </c>
     </row>
     <row r="63" spans="2:7" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="B63" s="9">
+      <c r="B63" s="8">
         <v>61</v>
       </c>
-      <c r="C63" s="10" t="s">
+      <c r="C63" s="9" t="s">
         <v>190</v>
       </c>
-      <c r="D63" s="9" t="s">
+      <c r="D63" s="8" t="s">
         <v>188</v>
       </c>
-      <c r="E63" s="9" t="s">
+      <c r="E63" s="8" t="s">
         <v>191</v>
       </c>
-      <c r="F63" s="12">
+      <c r="F63" s="11">
         <v>40305</v>
       </c>
-      <c r="G63" s="9" t="s">
+      <c r="G63" s="8" t="s">
         <v>70</v>
       </c>
     </row>
     <row r="64" spans="2:7" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="B64" s="9">
+      <c r="B64" s="8">
         <v>62</v>
       </c>
-      <c r="C64" s="10" t="s">
+      <c r="C64" s="9" t="s">
         <v>192</v>
       </c>
-      <c r="D64" s="9" t="s">
+      <c r="D64" s="8" t="s">
         <v>188</v>
       </c>
-      <c r="E64" s="9" t="s">
+      <c r="E64" s="8" t="s">
         <v>193</v>
       </c>
-      <c r="F64" s="11">
+      <c r="F64" s="10">
         <v>46302</v>
       </c>
-      <c r="G64" s="9" t="s">
+      <c r="G64" s="8" t="s">
         <v>70</v>
       </c>
     </row>
     <row r="65" spans="2:7" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="B65" s="9">
+      <c r="B65" s="8">
         <v>63</v>
       </c>
-      <c r="C65" s="10" t="s">
+      <c r="C65" s="9" t="s">
         <v>194</v>
       </c>
-      <c r="D65" s="9" t="s">
+      <c r="D65" s="8" t="s">
         <v>195</v>
       </c>
-      <c r="E65" s="9" t="s">
+      <c r="E65" s="8" t="s">
         <v>196</v>
       </c>
-      <c r="F65" s="12">
+      <c r="F65" s="11">
         <v>40305</v>
       </c>
-      <c r="G65" s="9" t="s">
+      <c r="G65" s="8" t="s">
         <v>70</v>
       </c>
     </row>
     <row r="66" spans="2:7" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="B66" s="9">
+      <c r="B66" s="8">
         <v>64</v>
       </c>
-      <c r="C66" s="10" t="s">
+      <c r="C66" s="9" t="s">
         <v>197</v>
       </c>
-      <c r="D66" s="9" t="s">
+      <c r="D66" s="8" t="s">
         <v>195</v>
       </c>
-      <c r="E66" s="9" t="s">
+      <c r="E66" s="8" t="s">
         <v>198</v>
       </c>
-      <c r="F66" s="12">
+      <c r="F66" s="11">
         <v>40305</v>
       </c>
-      <c r="G66" s="9" t="s">
+      <c r="G66" s="8" t="s">
         <v>70</v>
       </c>
     </row>
     <row r="67" spans="2:7" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="B67" s="9">
+      <c r="B67" s="8">
         <v>65</v>
       </c>
-      <c r="C67" s="9" t="s">
+      <c r="C67" s="8" t="s">
         <v>199</v>
       </c>
-      <c r="D67" s="9" t="s">
+      <c r="D67" s="8" t="s">
         <v>64</v>
       </c>
-      <c r="E67" s="12">
+      <c r="E67" s="11">
         <v>40305</v>
       </c>
-      <c r="F67" s="9" t="s">
+      <c r="F67" s="8" t="s">
         <v>70</v>
       </c>
     </row>
     <row r="68" spans="2:7" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="B68" s="9">
+      <c r="B68" s="8">
         <v>66</v>
       </c>
-      <c r="C68" s="9" t="s">
+      <c r="C68" s="8" t="s">
         <v>200</v>
       </c>
-      <c r="D68" s="9" t="s">
+      <c r="D68" s="8" t="s">
         <v>64</v>
       </c>
-      <c r="E68" s="11">
+      <c r="E68" s="10">
         <v>46302</v>
       </c>
-      <c r="F68" s="9" t="s">
+      <c r="F68" s="8" t="s">
         <v>70</v>
       </c>
     </row>
     <row r="69" spans="2:7" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="B69" s="9">
+      <c r="B69" s="8">
         <v>67</v>
       </c>
-      <c r="C69" s="9" t="s">
+      <c r="C69" s="8" t="s">
         <v>201</v>
       </c>
-      <c r="D69" s="9" t="s">
+      <c r="D69" s="8" t="s">
         <v>64</v>
       </c>
-      <c r="E69" s="11">
+      <c r="E69" s="10">
         <v>46302</v>
       </c>
-      <c r="F69" s="9" t="s">
+      <c r="F69" s="8" t="s">
         <v>70</v>
       </c>
     </row>
     <row r="70" spans="2:7" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="B70" s="9">
+      <c r="B70" s="8">
         <v>68</v>
       </c>
-      <c r="C70" s="9" t="s">
+      <c r="C70" s="8" t="s">
         <v>202</v>
       </c>
-      <c r="D70" s="9" t="s">
+      <c r="D70" s="8" t="s">
         <v>64</v>
       </c>
-      <c r="E70" s="11">
+      <c r="E70" s="10">
         <v>46302</v>
       </c>
-      <c r="F70" s="9" t="s">
+      <c r="F70" s="8" t="s">
         <v>70</v>
       </c>
     </row>
     <row r="71" spans="2:7" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="B71" s="9">
+      <c r="B71" s="8">
         <v>69</v>
       </c>
-      <c r="C71" s="9" t="s">
+      <c r="C71" s="8" t="s">
         <v>203</v>
       </c>
-      <c r="D71" s="9" t="s">
+      <c r="D71" s="8" t="s">
         <v>64</v>
       </c>
-      <c r="E71" s="11">
+      <c r="E71" s="10">
         <v>46302</v>
       </c>
-      <c r="F71" s="9" t="s">
+      <c r="F71" s="8" t="s">
         <v>70</v>
       </c>
     </row>
     <row r="72" spans="2:7" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="B72" s="9">
+      <c r="B72" s="8">
         <v>70</v>
       </c>
-      <c r="C72" s="9" t="s">
+      <c r="C72" s="8" t="s">
         <v>204</v>
       </c>
-      <c r="D72" s="9" t="s">
+      <c r="D72" s="8" t="s">
         <v>64</v>
       </c>
-      <c r="E72" s="12">
+      <c r="E72" s="11">
         <v>40304</v>
       </c>
-      <c r="F72" s="9" t="s">
+      <c r="F72" s="8" t="s">
         <v>118</v>
       </c>
     </row>
     <row r="73" spans="2:7" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="B73" s="9">
+      <c r="B73" s="8">
         <v>71</v>
       </c>
-      <c r="C73" s="9" t="s">
+      <c r="C73" s="8" t="s">
         <v>205</v>
       </c>
-      <c r="D73" s="9" t="s">
+      <c r="D73" s="8" t="s">
         <v>64</v>
       </c>
-      <c r="E73" s="12">
+      <c r="E73" s="11">
         <v>40304</v>
       </c>
-      <c r="F73" s="9" t="s">
+      <c r="F73" s="8" t="s">
         <v>118</v>
       </c>
     </row>
     <row r="74" spans="2:7" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="B74" s="9">
+      <c r="B74" s="8">
         <v>72</v>
       </c>
-      <c r="C74" s="9" t="s">
+      <c r="C74" s="8" t="s">
         <v>54</v>
       </c>
-      <c r="D74" s="9" t="s">
+      <c r="D74" s="8" t="s">
         <v>188</v>
       </c>
-      <c r="E74" s="12">
+      <c r="E74" s="11">
         <v>40304</v>
       </c>
-      <c r="F74" s="9" t="s">
+      <c r="F74" s="8" t="s">
         <v>118</v>
       </c>
     </row>
     <row r="75" spans="2:7" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="B75" s="9">
+      <c r="B75" s="8">
         <v>73</v>
       </c>
-      <c r="C75" s="9" t="s">
+      <c r="C75" s="8" t="s">
         <v>206</v>
       </c>
-      <c r="D75" s="9" t="s">
+      <c r="D75" s="8" t="s">
         <v>76</v>
       </c>
-      <c r="E75" s="12">
+      <c r="E75" s="11">
         <v>40304</v>
       </c>
-      <c r="F75" s="9" t="s">
+      <c r="F75" s="8" t="s">
         <v>118</v>
       </c>
     </row>
     <row r="76" spans="2:7" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="B76" s="9">
+      <c r="B76" s="8">
         <v>74</v>
       </c>
-      <c r="C76" s="9" t="s">
+      <c r="C76" s="8" t="s">
         <v>207</v>
       </c>
-      <c r="D76" s="9" t="s">
+      <c r="D76" s="8" t="s">
         <v>208</v>
       </c>
-      <c r="E76" s="11">
+      <c r="E76" s="10">
         <v>46302</v>
       </c>
-      <c r="F76" s="9" t="s">
+      <c r="F76" s="8" t="s">
         <v>70</v>
       </c>
     </row>
     <row r="77" spans="2:7" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="B77" s="9">
+      <c r="B77" s="8">
         <v>75</v>
       </c>
-      <c r="C77" s="9" t="s">
+      <c r="C77" s="8" t="s">
         <v>209</v>
       </c>
-      <c r="D77" s="9" t="s">
+      <c r="D77" s="8" t="s">
         <v>208</v>
       </c>
-      <c r="E77" s="11">
+      <c r="E77" s="10">
         <v>46302</v>
       </c>
-      <c r="F77" s="9" t="s">
+      <c r="F77" s="8" t="s">
         <v>70</v>
       </c>
     </row>
     <row r="78" spans="2:7" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="B78" s="9">
+      <c r="B78" s="8">
         <v>76</v>
       </c>
-      <c r="C78" s="9" t="s">
+      <c r="C78" s="8" t="s">
         <v>210</v>
       </c>
-      <c r="D78" s="9" t="s">
+      <c r="D78" s="8" t="s">
         <v>208</v>
       </c>
-      <c r="E78" s="12">
+      <c r="E78" s="11">
         <v>40304</v>
       </c>
-      <c r="F78" s="9" t="s">
+      <c r="F78" s="8" t="s">
         <v>70</v>
       </c>
     </row>
     <row r="79" spans="2:7" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="B79" s="9">
+      <c r="B79" s="8">
         <v>77</v>
       </c>
-      <c r="C79" s="9" t="s">
+      <c r="C79" s="8" t="s">
         <v>211</v>
       </c>
-      <c r="D79" s="9" t="s">
+      <c r="D79" s="8" t="s">
         <v>208</v>
       </c>
-      <c r="E79" s="12">
+      <c r="E79" s="11">
         <v>40304</v>
       </c>
-      <c r="F79" s="9" t="s">
+      <c r="F79" s="8" t="s">
         <v>70</v>
       </c>
     </row>
     <row r="80" spans="2:7" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="B80" s="9">
+      <c r="B80" s="8">
         <v>78</v>
       </c>
-      <c r="C80" s="9" t="s">
+      <c r="C80" s="8" t="s">
         <v>212</v>
       </c>
-      <c r="D80" s="9" t="s">
+      <c r="D80" s="8" t="s">
         <v>208</v>
       </c>
-      <c r="E80" s="12">
+      <c r="E80" s="11">
         <v>40304</v>
       </c>
-      <c r="F80" s="9" t="s">
+      <c r="F80" s="8" t="s">
         <v>70</v>
       </c>
     </row>
     <row r="81" spans="2:6" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="B81" s="9">
+      <c r="B81" s="8">
         <v>79</v>
       </c>
-      <c r="C81" s="9" t="s">
+      <c r="C81" s="8" t="s">
         <v>213</v>
       </c>
-      <c r="D81" s="9" t="s">
+      <c r="D81" s="8" t="s">
         <v>94</v>
       </c>
-      <c r="E81" s="11">
+      <c r="E81" s="10">
         <v>46302</v>
       </c>
-      <c r="F81" s="9" t="s">
+      <c r="F81" s="8" t="s">
         <v>70</v>
       </c>
     </row>
     <row r="82" spans="2:6" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="B82" s="9">
+      <c r="B82" s="8">
         <v>80</v>
       </c>
-      <c r="C82" s="9" t="s">
+      <c r="C82" s="8" t="s">
         <v>214</v>
       </c>
-      <c r="D82" s="9" t="s">
+      <c r="D82" s="8" t="s">
         <v>94</v>
       </c>
-      <c r="E82" s="11">
+      <c r="E82" s="10">
         <v>46302</v>
       </c>
-      <c r="F82" s="9" t="s">
+      <c r="F82" s="8" t="s">
         <v>70</v>
       </c>
     </row>
     <row r="83" spans="2:6" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="B83" s="9">
+      <c r="B83" s="8">
         <v>81</v>
       </c>
-      <c r="C83" s="9" t="s">
+      <c r="C83" s="8" t="s">
         <v>215</v>
       </c>
-      <c r="D83" s="9" t="s">
+      <c r="D83" s="8" t="s">
         <v>94</v>
       </c>
-      <c r="E83" s="12">
+      <c r="E83" s="11">
         <v>40304</v>
       </c>
-      <c r="F83" s="9" t="s">
+      <c r="F83" s="8" t="s">
         <v>70</v>
       </c>
     </row>
     <row r="84" spans="2:6" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="B84" s="9">
+      <c r="B84" s="8">
         <v>82</v>
       </c>
-      <c r="C84" s="9" t="s">
+      <c r="C84" s="8" t="s">
         <v>216</v>
       </c>
-      <c r="D84" s="9" t="s">
+      <c r="D84" s="8" t="s">
         <v>94</v>
       </c>
-      <c r="E84" s="12">
+      <c r="E84" s="11">
         <v>40304</v>
       </c>
-      <c r="F84" s="9" t="s">
+      <c r="F84" s="8" t="s">
         <v>70</v>
       </c>
     </row>
     <row r="85" spans="2:6" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="B85" s="9">
+      <c r="B85" s="8">
         <v>83</v>
       </c>
-      <c r="C85" s="9" t="s">
+      <c r="C85" s="8" t="s">
         <v>217</v>
       </c>
-      <c r="D85" s="9" t="s">
+      <c r="D85" s="8" t="s">
         <v>68</v>
       </c>
-      <c r="E85" s="11">
+      <c r="E85" s="10">
         <v>46302</v>
       </c>
-      <c r="F85" s="9" t="s">
+      <c r="F85" s="8" t="s">
         <v>70</v>
       </c>
     </row>
     <row r="86" spans="2:6" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="B86" s="9">
+      <c r="B86" s="8">
         <v>84</v>
       </c>
-      <c r="C86" s="9" t="s">
+      <c r="C86" s="8" t="s">
         <v>218</v>
       </c>
-      <c r="D86" s="9" t="s">
+      <c r="D86" s="8" t="s">
         <v>68</v>
       </c>
-      <c r="E86" s="12">
+      <c r="E86" s="11">
         <v>40304</v>
       </c>
-      <c r="F86" s="9" t="s">
+      <c r="F86" s="8" t="s">
         <v>70</v>
       </c>
     </row>
     <row r="87" spans="2:6" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="B87" s="9">
+      <c r="B87" s="8">
         <v>85</v>
       </c>
-      <c r="C87" s="9" t="s">
+      <c r="C87" s="8" t="s">
         <v>219</v>
       </c>
-      <c r="D87" s="9" t="s">
+      <c r="D87" s="8" t="s">
         <v>68</v>
       </c>
-      <c r="E87" s="12">
+      <c r="E87" s="11">
         <v>40304</v>
       </c>
-      <c r="F87" s="9" t="s">
+      <c r="F87" s="8" t="s">
         <v>70</v>
       </c>
     </row>
     <row r="88" spans="2:6" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="B88" s="9">
+      <c r="B88" s="8">
         <v>86</v>
       </c>
-      <c r="C88" s="9" t="s">
+      <c r="C88" s="8" t="s">
         <v>220</v>
       </c>
-      <c r="D88" s="9" t="s">
+      <c r="D88" s="8" t="s">
         <v>68</v>
       </c>
-      <c r="E88" s="12">
+      <c r="E88" s="11">
         <v>40304</v>
       </c>
-      <c r="F88" s="9" t="s">
+      <c r="F88" s="8" t="s">
         <v>70</v>
       </c>
     </row>
     <row r="89" spans="2:6" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="B89" s="9">
+      <c r="B89" s="8">
         <v>87</v>
       </c>
-      <c r="C89" s="9" t="s">
+      <c r="C89" s="8" t="s">
         <v>221</v>
       </c>
-      <c r="D89" s="9" t="s">
+      <c r="D89" s="8" t="s">
         <v>68</v>
       </c>
-      <c r="E89" s="11">
+      <c r="E89" s="10">
         <v>46301</v>
       </c>
-      <c r="F89" s="9" t="s">
+      <c r="F89" s="8" t="s">
         <v>118</v>
       </c>
     </row>
     <row r="90" spans="2:6" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="B90" s="9">
+      <c r="B90" s="8">
         <v>88</v>
       </c>
-      <c r="C90" s="9" t="s">
+      <c r="C90" s="8" t="s">
         <v>222</v>
       </c>
-      <c r="D90" s="9" t="s">
+      <c r="D90" s="8" t="s">
         <v>68</v>
       </c>
-      <c r="E90" s="12">
+      <c r="E90" s="11">
         <v>40304</v>
       </c>
-      <c r="F90" s="9" t="s">
+      <c r="F90" s="8" t="s">
         <v>118</v>
       </c>
     </row>
     <row r="91" spans="2:6" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="B91" s="9">
+      <c r="B91" s="8">
         <v>89</v>
       </c>
-      <c r="C91" s="9" t="s">
+      <c r="C91" s="8" t="s">
         <v>223</v>
       </c>
-      <c r="D91" s="9" t="s">
+      <c r="D91" s="8" t="s">
         <v>68</v>
       </c>
-      <c r="E91" s="12">
+      <c r="E91" s="11">
         <v>40304</v>
       </c>
-      <c r="F91" s="9" t="s">
+      <c r="F91" s="8" t="s">
         <v>70</v>
       </c>
     </row>
     <row r="92" spans="2:6" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="B92" s="9">
+      <c r="B92" s="8">
         <v>90</v>
       </c>
-      <c r="C92" s="9" t="s">
+      <c r="C92" s="8" t="s">
         <v>224</v>
       </c>
-      <c r="D92" s="9" t="s">
+      <c r="D92" s="8" t="s">
         <v>68</v>
       </c>
-      <c r="E92" s="12">
+      <c r="E92" s="11">
         <v>40304</v>
       </c>
-      <c r="F92" s="9" t="s">
+      <c r="F92" s="8" t="s">
         <v>70</v>
       </c>
     </row>
     <row r="93" spans="2:6" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="B93" s="9">
+      <c r="B93" s="8">
         <v>91</v>
       </c>
-      <c r="C93" s="9" t="s">
+      <c r="C93" s="8" t="s">
         <v>225</v>
       </c>
-      <c r="D93" s="9" t="s">
+      <c r="D93" s="8" t="s">
         <v>76</v>
       </c>
-      <c r="E93" s="12">
+      <c r="E93" s="11">
         <v>40304</v>
       </c>
-      <c r="F93" s="9" t="s">
+      <c r="F93" s="8" t="s">
         <v>118</v>
       </c>
     </row>
     <row r="94" spans="2:6" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="B94" s="9">
+      <c r="B94" s="8">
         <v>92</v>
       </c>
-      <c r="C94" s="9" t="s">
+      <c r="C94" s="8" t="s">
         <v>226</v>
       </c>
-      <c r="D94" s="9" t="s">
+      <c r="D94" s="8" t="s">
         <v>76</v>
       </c>
-      <c r="E94" s="12">
+      <c r="E94" s="11">
         <v>40304</v>
       </c>
-      <c r="F94" s="9" t="s">
+      <c r="F94" s="8" t="s">
         <v>118</v>
       </c>
     </row>
     <row r="95" spans="2:6" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="B95" s="9">
+      <c r="B95" s="8">
         <v>93</v>
       </c>
-      <c r="C95" s="9" t="s">
+      <c r="C95" s="8" t="s">
         <v>227</v>
       </c>
-      <c r="D95" s="9" t="s">
+      <c r="D95" s="8" t="s">
         <v>76</v>
       </c>
-      <c r="E95" s="12">
+      <c r="E95" s="11">
         <v>40304</v>
       </c>
-      <c r="F95" s="9" t="s">
+      <c r="F95" s="8" t="s">
         <v>118</v>
       </c>
     </row>
     <row r="96" spans="2:6" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="B96" s="9">
+      <c r="B96" s="8">
         <v>94</v>
       </c>
-      <c r="C96" s="9" t="s">
+      <c r="C96" s="8" t="s">
         <v>228</v>
       </c>
-      <c r="D96" s="9" t="s">
+      <c r="D96" s="8" t="s">
         <v>76</v>
       </c>
-      <c r="E96" s="12">
+      <c r="E96" s="11">
         <v>40304</v>
       </c>
-      <c r="F96" s="9" t="s">
+      <c r="F96" s="8" t="s">
         <v>70</v>
       </c>
     </row>
     <row r="97" spans="2:6" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="B97" s="9">
+      <c r="B97" s="8">
         <v>95</v>
       </c>
-      <c r="C97" s="9" t="s">
+      <c r="C97" s="8" t="s">
         <v>229</v>
       </c>
-      <c r="D97" s="9" t="s">
+      <c r="D97" s="8" t="s">
         <v>76</v>
       </c>
-      <c r="E97" s="12">
+      <c r="E97" s="11">
         <v>40304</v>
       </c>
-      <c r="F97" s="9" t="s">
+      <c r="F97" s="8" t="s">
         <v>118</v>
       </c>
     </row>
     <row r="98" spans="2:6" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="B98" s="9">
+      <c r="B98" s="8">
         <v>96</v>
       </c>
-      <c r="C98" s="9" t="s">
+      <c r="C98" s="8" t="s">
         <v>230</v>
       </c>
-      <c r="D98" s="9" t="s">
+      <c r="D98" s="8" t="s">
         <v>76</v>
       </c>
-      <c r="E98" s="12">
+      <c r="E98" s="11">
         <v>40304</v>
       </c>
-      <c r="F98" s="9" t="s">
+      <c r="F98" s="8" t="s">
         <v>118</v>
       </c>
     </row>
     <row r="99" spans="2:6" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="B99" s="9">
+      <c r="B99" s="8">
         <v>97</v>
       </c>
-      <c r="C99" s="9" t="s">
+      <c r="C99" s="8" t="s">
         <v>231</v>
       </c>
-      <c r="D99" s="9" t="s">
+      <c r="D99" s="8" t="s">
         <v>76</v>
       </c>
-      <c r="E99" s="12">
+      <c r="E99" s="11">
         <v>40304</v>
       </c>
-      <c r="F99" s="9" t="s">
+      <c r="F99" s="8" t="s">
         <v>118</v>
       </c>
     </row>
     <row r="100" spans="2:6" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="B100" s="9">
+      <c r="B100" s="8">
         <v>98</v>
       </c>
-      <c r="C100" s="9" t="s">
+      <c r="C100" s="8" t="s">
         <v>232</v>
       </c>
-      <c r="D100" s="9" t="s">
+      <c r="D100" s="8" t="s">
         <v>76</v>
       </c>
-      <c r="E100" s="12">
+      <c r="E100" s="11">
         <v>40304</v>
       </c>
-      <c r="F100" s="9" t="s">
+      <c r="F100" s="8" t="s">
         <v>118</v>
       </c>
     </row>
     <row r="101" spans="2:6" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="B101" s="9">
+      <c r="B101" s="8">
         <v>99</v>
       </c>
-      <c r="C101" s="9" t="s">
+      <c r="C101" s="8" t="s">
         <v>233</v>
       </c>
-      <c r="D101" s="9" t="s">
+      <c r="D101" s="8" t="s">
         <v>76</v>
       </c>
-      <c r="E101" s="12">
+      <c r="E101" s="11">
         <v>40304</v>
       </c>
-      <c r="F101" s="9" t="s">
+      <c r="F101" s="8" t="s">
         <v>118</v>
       </c>
     </row>
     <row r="102" spans="2:6" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="B102" s="9">
+      <c r="B102" s="8">
         <v>100</v>
       </c>
-      <c r="C102" s="9" t="s">
+      <c r="C102" s="8" t="s">
         <v>234</v>
       </c>
-      <c r="D102" s="9" t="s">
+      <c r="D102" s="8" t="s">
         <v>76</v>
       </c>
-      <c r="E102" s="12">
+      <c r="E102" s="11">
         <v>40304</v>
       </c>
-      <c r="F102" s="9" t="s">
+      <c r="F102" s="8" t="s">
         <v>118</v>
       </c>
     </row>
     <row r="103" spans="2:6" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="B103" s="9">
+      <c r="B103" s="8">
         <v>101</v>
       </c>
-      <c r="C103" s="9" t="s">
+      <c r="C103" s="8" t="s">
         <v>235</v>
       </c>
-      <c r="D103" s="9" t="s">
+      <c r="D103" s="8" t="s">
         <v>89</v>
       </c>
-      <c r="E103" s="11">
+      <c r="E103" s="10">
         <v>46302</v>
       </c>
-      <c r="F103" s="9" t="s">
+      <c r="F103" s="8" t="s">
         <v>70</v>
       </c>
     </row>
     <row r="104" spans="2:6" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="B104" s="9">
+      <c r="B104" s="8">
         <v>102</v>
       </c>
-      <c r="C104" s="9" t="s">
+      <c r="C104" s="8" t="s">
         <v>236</v>
       </c>
-      <c r="D104" s="9" t="s">
+      <c r="D104" s="8" t="s">
         <v>89</v>
       </c>
-      <c r="E104" s="12">
+      <c r="E104" s="11">
         <v>40304</v>
       </c>
-      <c r="F104" s="9" t="s">
+      <c r="F104" s="8" t="s">
         <v>118</v>
       </c>
     </row>
     <row r="105" spans="2:6" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="B105" s="9">
+      <c r="B105" s="8">
         <v>103</v>
       </c>
-      <c r="C105" s="9" t="s">
+      <c r="C105" s="8" t="s">
         <v>237</v>
       </c>
-      <c r="D105" s="9" t="s">
+      <c r="D105" s="8" t="s">
         <v>188</v>
       </c>
-      <c r="E105" s="11">
+      <c r="E105" s="10">
         <v>46302</v>
       </c>
-      <c r="F105" s="9" t="s">
+      <c r="F105" s="8" t="s">
         <v>70</v>
       </c>
     </row>
     <row r="106" spans="2:6" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="B106" s="9">
+      <c r="B106" s="8">
         <v>104</v>
       </c>
-      <c r="C106" s="9" t="s">
+      <c r="C106" s="8" t="s">
         <v>238</v>
       </c>
-      <c r="D106" s="9" t="s">
+      <c r="D106" s="8" t="s">
         <v>188</v>
       </c>
-      <c r="E106" s="11">
+      <c r="E106" s="10">
         <v>46302</v>
       </c>
-      <c r="F106" s="9" t="s">
+      <c r="F106" s="8" t="s">
         <v>70</v>
       </c>
     </row>
     <row r="107" spans="2:6" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="B107" s="9">
+      <c r="B107" s="8">
         <v>105</v>
       </c>
-      <c r="C107" s="9" t="s">
+      <c r="C107" s="8" t="s">
         <v>239</v>
       </c>
-      <c r="D107" s="9" t="s">
+      <c r="D107" s="8" t="s">
         <v>188</v>
       </c>
-      <c r="E107" s="11">
+      <c r="E107" s="10">
         <v>46302</v>
       </c>
-      <c r="F107" s="9" t="s">
+      <c r="F107" s="8" t="s">
         <v>70</v>
       </c>
     </row>
     <row r="108" spans="2:6" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="B108" s="9">
+      <c r="B108" s="8">
         <v>106</v>
       </c>
-      <c r="C108" s="9" t="s">
+      <c r="C108" s="8" t="s">
         <v>240</v>
       </c>
-      <c r="D108" s="9" t="s">
+      <c r="D108" s="8" t="s">
         <v>188</v>
       </c>
-      <c r="E108" s="11">
+      <c r="E108" s="10">
         <v>46302</v>
       </c>
-      <c r="F108" s="9" t="s">
+      <c r="F108" s="8" t="s">
         <v>70</v>
       </c>
     </row>
     <row r="109" spans="2:6" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="B109" s="9">
+      <c r="B109" s="8">
         <v>107</v>
       </c>
-      <c r="C109" s="9" t="s">
+      <c r="C109" s="8" t="s">
         <v>241</v>
       </c>
-      <c r="D109" s="9" t="s">
+      <c r="D109" s="8" t="s">
         <v>188</v>
       </c>
-      <c r="E109" s="11">
+      <c r="E109" s="10">
         <v>46302</v>
       </c>
-      <c r="F109" s="9" t="s">
+      <c r="F109" s="8" t="s">
         <v>70</v>
       </c>
     </row>
     <row r="110" spans="2:6" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="B110" s="9">
+      <c r="B110" s="8">
         <v>108</v>
       </c>
-      <c r="C110" s="9" t="s">
+      <c r="C110" s="8" t="s">
         <v>242</v>
       </c>
-      <c r="D110" s="9" t="s">
+      <c r="D110" s="8" t="s">
         <v>188</v>
       </c>
-      <c r="E110" s="11">
+      <c r="E110" s="10">
         <v>46302</v>
       </c>
-      <c r="F110" s="9" t="s">
+      <c r="F110" s="8" t="s">
         <v>70</v>
       </c>
     </row>
     <row r="111" spans="2:6" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="B111" s="9">
+      <c r="B111" s="8">
         <v>109</v>
       </c>
-      <c r="C111" s="9" t="s">
+      <c r="C111" s="8" t="s">
         <v>243</v>
       </c>
-      <c r="D111" s="9" t="s">
+      <c r="D111" s="8" t="s">
         <v>89</v>
       </c>
-      <c r="E111" s="12">
+      <c r="E111" s="11">
         <v>40303</v>
       </c>
-      <c r="F111" s="9" t="s">
+      <c r="F111" s="8" t="s">
         <v>118</v>
       </c>
     </row>
     <row r="112" spans="2:6" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="B112" s="9">
+      <c r="B112" s="8">
         <v>110</v>
       </c>
-      <c r="C112" s="9" t="s">
+      <c r="C112" s="8" t="s">
         <v>244</v>
       </c>
-      <c r="D112" s="9" t="s">
+      <c r="D112" s="8" t="s">
         <v>64</v>
       </c>
-      <c r="E112" s="12">
+      <c r="E112" s="11">
         <v>40304</v>
       </c>
-      <c r="F112" s="9" t="s">
+      <c r="F112" s="8" t="s">
         <v>118</v>
       </c>
     </row>
     <row r="113" spans="2:6" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="B113" s="9">
+      <c r="B113" s="8">
         <v>111</v>
       </c>
-      <c r="C113" s="9" t="s">
+      <c r="C113" s="8" t="s">
         <v>245</v>
       </c>
-      <c r="D113" s="9" t="s">
+      <c r="D113" s="8" t="s">
         <v>64</v>
       </c>
-      <c r="E113" s="12">
+      <c r="E113" s="11">
         <v>40303</v>
       </c>
-      <c r="F113" s="9" t="s">
+      <c r="F113" s="8" t="s">
         <v>118</v>
       </c>
     </row>
     <row r="114" spans="2:6" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="B114" s="9">
+      <c r="B114" s="8">
         <v>112</v>
       </c>
-      <c r="C114" s="9" t="s">
+      <c r="C114" s="8" t="s">
         <v>246</v>
       </c>
-      <c r="D114" s="9" t="s">
+      <c r="D114" s="8" t="s">
         <v>64</v>
       </c>
-      <c r="E114" s="11">
+      <c r="E114" s="10">
         <v>46301</v>
       </c>
-      <c r="F114" s="9" t="s">
+      <c r="F114" s="8" t="s">
         <v>118</v>
       </c>
     </row>
     <row r="115" spans="2:6" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="B115" s="9">
+      <c r="B115" s="8">
         <v>113</v>
       </c>
-      <c r="C115" s="9" t="s">
+      <c r="C115" s="8" t="s">
         <v>247</v>
       </c>
-      <c r="D115" s="9" t="s">
+      <c r="D115" s="8" t="s">
         <v>64</v>
       </c>
-      <c r="E115" s="11">
+      <c r="E115" s="10">
         <v>46301</v>
       </c>
-      <c r="F115" s="9" t="s">
+      <c r="F115" s="8" t="s">
         <v>118</v>
       </c>
     </row>
     <row r="116" spans="2:6" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="B116" s="9">
+      <c r="B116" s="8">
         <v>114</v>
       </c>
-      <c r="C116" s="9" t="s">
+      <c r="C116" s="8" t="s">
         <v>248</v>
       </c>
-      <c r="D116" s="9" t="s">
+      <c r="D116" s="8" t="s">
         <v>208</v>
       </c>
-      <c r="E116" s="12">
+      <c r="E116" s="11">
         <v>40303</v>
       </c>
-      <c r="F116" s="9" t="s">
+      <c r="F116" s="8" t="s">
         <v>118</v>
       </c>
     </row>
     <row r="117" spans="2:6" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="B117" s="9">
+      <c r="B117" s="8">
         <v>115</v>
       </c>
-      <c r="C117" s="9" t="s">
+      <c r="C117" s="8" t="s">
         <v>249</v>
       </c>
-      <c r="D117" s="9" t="s">
+      <c r="D117" s="8" t="s">
         <v>208</v>
       </c>
-      <c r="E117" s="11">
+      <c r="E117" s="10">
         <v>46300</v>
       </c>
-      <c r="F117" s="9" t="s">
+      <c r="F117" s="8" t="s">
         <v>118</v>
       </c>
     </row>
     <row r="118" spans="2:6" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="B118" s="9">
+      <c r="B118" s="8">
         <v>116</v>
       </c>
-      <c r="C118" s="9" t="s">
+      <c r="C118" s="8" t="s">
         <v>250</v>
       </c>
-      <c r="D118" s="9" t="s">
+      <c r="D118" s="8" t="s">
         <v>208</v>
       </c>
-      <c r="E118" s="11">
+      <c r="E118" s="10">
         <v>46301</v>
       </c>
-      <c r="F118" s="9" t="s">
+      <c r="F118" s="8" t="s">
         <v>118</v>
       </c>
     </row>
     <row r="119" spans="2:6" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="B119" s="9">
+      <c r="B119" s="8">
         <v>117</v>
       </c>
-      <c r="C119" s="9" t="s">
+      <c r="C119" s="8" t="s">
         <v>251</v>
       </c>
-      <c r="D119" s="9" t="s">
+      <c r="D119" s="8" t="s">
         <v>208</v>
       </c>
-      <c r="E119" s="11">
+      <c r="E119" s="10">
         <v>46300</v>
       </c>
-      <c r="F119" s="9" t="s">
+      <c r="F119" s="8" t="s">
         <v>118</v>
       </c>
     </row>
     <row r="120" spans="2:6" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="B120" s="9">
+      <c r="B120" s="8">
         <v>118</v>
       </c>
-      <c r="C120" s="9" t="s">
+      <c r="C120" s="8" t="s">
         <v>252</v>
       </c>
-      <c r="D120" s="9" t="s">
+      <c r="D120" s="8" t="s">
         <v>208</v>
       </c>
-      <c r="E120" s="11">
+      <c r="E120" s="10">
         <v>46300</v>
       </c>
-      <c r="F120" s="9" t="s">
+      <c r="F120" s="8" t="s">
         <v>118</v>
       </c>
     </row>
     <row r="121" spans="2:6" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="B121" s="9">
+      <c r="B121" s="8">
         <v>119</v>
       </c>
-      <c r="C121" s="9" t="s">
+      <c r="C121" s="8" t="s">
         <v>253</v>
       </c>
-      <c r="D121" s="9" t="s">
+      <c r="D121" s="8" t="s">
         <v>208</v>
       </c>
-      <c r="E121" s="11">
+      <c r="E121" s="10">
         <v>46300</v>
       </c>
-      <c r="F121" s="9" t="s">
+      <c r="F121" s="8" t="s">
         <v>254</v>
       </c>
     </row>
     <row r="122" spans="2:6" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="B122" s="9">
+      <c r="B122" s="8">
         <v>120</v>
       </c>
-      <c r="C122" s="9" t="s">
+      <c r="C122" s="8" t="s">
         <v>255</v>
       </c>
-      <c r="D122" s="9" t="s">
+      <c r="D122" s="8" t="s">
         <v>94</v>
       </c>
-      <c r="E122" s="12">
+      <c r="E122" s="11">
         <v>40304</v>
       </c>
-      <c r="F122" s="9" t="s">
+      <c r="F122" s="8" t="s">
         <v>118</v>
       </c>
     </row>
     <row r="123" spans="2:6" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="B123" s="9">
+      <c r="B123" s="8">
         <v>121</v>
       </c>
-      <c r="C123" s="9" t="s">
+      <c r="C123" s="8" t="s">
         <v>256</v>
       </c>
-      <c r="D123" s="9" t="s">
+      <c r="D123" s="8" t="s">
         <v>94</v>
       </c>
-      <c r="E123" s="11">
+      <c r="E123" s="10">
         <v>46301</v>
       </c>
-      <c r="F123" s="9" t="s">
+      <c r="F123" s="8" t="s">
         <v>118</v>
       </c>
     </row>
     <row r="124" spans="2:6" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="B124" s="9">
+      <c r="B124" s="8">
         <v>122</v>
       </c>
-      <c r="C124" s="9" t="s">
+      <c r="C124" s="8" t="s">
         <v>257</v>
       </c>
-      <c r="D124" s="9" t="s">
+      <c r="D124" s="8" t="s">
         <v>94</v>
       </c>
-      <c r="E124" s="11">
+      <c r="E124" s="10">
         <v>46301</v>
       </c>
-      <c r="F124" s="9" t="s">
+      <c r="F124" s="8" t="s">
         <v>118</v>
       </c>
     </row>
     <row r="125" spans="2:6" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="B125" s="9">
+      <c r="B125" s="8">
         <v>123</v>
       </c>
-      <c r="C125" s="9" t="s">
+      <c r="C125" s="8" t="s">
         <v>258</v>
       </c>
-      <c r="D125" s="9" t="s">
+      <c r="D125" s="8" t="s">
         <v>94</v>
       </c>
-      <c r="E125" s="12">
+      <c r="E125" s="11">
         <v>40303</v>
       </c>
-      <c r="F125" s="9" t="s">
+      <c r="F125" s="8" t="s">
         <v>118</v>
       </c>
     </row>
     <row r="126" spans="2:6" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="B126" s="9">
+      <c r="B126" s="8">
         <v>124</v>
       </c>
-      <c r="C126" s="9" t="s">
+      <c r="C126" s="8" t="s">
         <v>259</v>
       </c>
-      <c r="D126" s="9" t="s">
+      <c r="D126" s="8" t="s">
         <v>94</v>
       </c>
-      <c r="E126" s="11">
+      <c r="E126" s="10">
         <v>46300</v>
       </c>
-      <c r="F126" s="9" t="s">
+      <c r="F126" s="8" t="s">
         <v>118</v>
       </c>
     </row>
     <row r="127" spans="2:6" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="B127" s="9">
+      <c r="B127" s="8">
         <v>125</v>
       </c>
-      <c r="C127" s="9" t="s">
+      <c r="C127" s="8" t="s">
         <v>260</v>
       </c>
-      <c r="D127" s="9" t="s">
+      <c r="D127" s="8" t="s">
         <v>68</v>
       </c>
-      <c r="E127" s="12">
+      <c r="E127" s="11">
         <v>40303</v>
       </c>
-      <c r="F127" s="9" t="s">
+      <c r="F127" s="8" t="s">
         <v>118</v>
       </c>
     </row>
     <row r="128" spans="2:6" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="B128" s="9">
+      <c r="B128" s="8">
         <v>126</v>
       </c>
-      <c r="C128" s="9" t="s">
+      <c r="C128" s="8" t="s">
         <v>261</v>
       </c>
-      <c r="D128" s="9" t="s">
+      <c r="D128" s="8" t="s">
         <v>68</v>
       </c>
-      <c r="E128" s="11">
+      <c r="E128" s="10">
         <v>46301</v>
       </c>
-      <c r="F128" s="9" t="s">
+      <c r="F128" s="8" t="s">
         <v>118</v>
       </c>
     </row>
     <row r="129" spans="2:6" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="B129" s="9">
+      <c r="B129" s="8">
         <v>127</v>
       </c>
-      <c r="C129" s="9" t="s">
+      <c r="C129" s="8" t="s">
         <v>262</v>
       </c>
-      <c r="D129" s="9" t="s">
+      <c r="D129" s="8" t="s">
         <v>68</v>
       </c>
-      <c r="E129" s="11">
+      <c r="E129" s="10">
         <v>46301</v>
       </c>
-      <c r="F129" s="9" t="s">
+      <c r="F129" s="8" t="s">
         <v>118</v>
       </c>
     </row>
     <row r="130" spans="2:6" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="B130" s="9">
+      <c r="B130" s="8">
         <v>128</v>
       </c>
-      <c r="C130" s="9" t="s">
+      <c r="C130" s="8" t="s">
         <v>263</v>
       </c>
-      <c r="D130" s="9" t="s">
+      <c r="D130" s="8" t="s">
         <v>76</v>
       </c>
-      <c r="E130" s="11">
+      <c r="E130" s="10">
         <v>46300</v>
       </c>
-      <c r="F130" s="9" t="s">
+      <c r="F130" s="8" t="s">
         <v>118</v>
       </c>
     </row>
     <row r="131" spans="2:6" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="B131" s="9">
+      <c r="B131" s="8">
         <v>129</v>
       </c>
-      <c r="C131" s="9" t="s">
+      <c r="C131" s="8" t="s">
         <v>264</v>
       </c>
-      <c r="D131" s="9" t="s">
+      <c r="D131" s="8" t="s">
         <v>76</v>
       </c>
-      <c r="E131" s="12">
+      <c r="E131" s="11">
         <v>40303</v>
       </c>
-      <c r="F131" s="9" t="s">
+      <c r="F131" s="8" t="s">
         <v>118</v>
       </c>
     </row>
     <row r="132" spans="2:6" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="B132" s="9">
+      <c r="B132" s="8">
         <v>130</v>
       </c>
-      <c r="C132" s="9" t="s">
+      <c r="C132" s="8" t="s">
         <v>265</v>
       </c>
-      <c r="D132" s="9" t="s">
+      <c r="D132" s="8" t="s">
         <v>76</v>
       </c>
-      <c r="E132" s="12">
+      <c r="E132" s="11">
         <v>40303</v>
       </c>
-      <c r="F132" s="9" t="s">
+      <c r="F132" s="8" t="s">
         <v>118</v>
       </c>
     </row>
     <row r="133" spans="2:6" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="B133" s="9">
+      <c r="B133" s="8">
         <v>131</v>
       </c>
-      <c r="C133" s="9" t="s">
+      <c r="C133" s="8" t="s">
         <v>266</v>
       </c>
-      <c r="D133" s="9" t="s">
+      <c r="D133" s="8" t="s">
         <v>76</v>
       </c>
-      <c r="E133" s="12">
+      <c r="E133" s="11">
         <v>40303</v>
       </c>
-      <c r="F133" s="9" t="s">
+      <c r="F133" s="8" t="s">
         <v>118</v>
       </c>
     </row>
     <row r="134" spans="2:6" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="B134" s="9">
+      <c r="B134" s="8">
         <v>132</v>
       </c>
-      <c r="C134" s="9" t="s">
+      <c r="C134" s="8" t="s">
         <v>267</v>
       </c>
-      <c r="D134" s="9" t="s">
+      <c r="D134" s="8" t="s">
         <v>76</v>
       </c>
-      <c r="E134" s="11">
+      <c r="E134" s="10">
         <v>46301</v>
       </c>
-      <c r="F134" s="9" t="s">
+      <c r="F134" s="8" t="s">
         <v>118</v>
       </c>
     </row>
     <row r="135" spans="2:6" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="B135" s="9">
+      <c r="B135" s="8">
         <v>133</v>
       </c>
-      <c r="C135" s="9" t="s">
+      <c r="C135" s="8" t="s">
         <v>268</v>
       </c>
-      <c r="D135" s="9" t="s">
+      <c r="D135" s="8" t="s">
         <v>76</v>
       </c>
-      <c r="E135" s="11">
+      <c r="E135" s="10">
         <v>46301</v>
       </c>
-      <c r="F135" s="9" t="s">
+      <c r="F135" s="8" t="s">
         <v>118</v>
       </c>
     </row>
     <row r="136" spans="2:6" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="B136" s="9">
+      <c r="B136" s="8">
         <v>134</v>
       </c>
-      <c r="C136" s="9" t="s">
+      <c r="C136" s="8" t="s">
         <v>269</v>
       </c>
-      <c r="D136" s="9" t="s">
+      <c r="D136" s="8" t="s">
         <v>76</v>
       </c>
-      <c r="E136" s="11">
+      <c r="E136" s="10">
         <v>46301</v>
       </c>
-      <c r="F136" s="9" t="s">
+      <c r="F136" s="8" t="s">
         <v>118</v>
       </c>
     </row>
     <row r="137" spans="2:6" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="B137" s="9">
+      <c r="B137" s="8">
         <v>135</v>
       </c>
-      <c r="C137" s="9" t="s">
+      <c r="C137" s="8" t="s">
         <v>270</v>
       </c>
-      <c r="D137" s="9" t="s">
+      <c r="D137" s="8" t="s">
         <v>76</v>
       </c>
-      <c r="E137" s="12">
+      <c r="E137" s="11">
         <v>40303</v>
       </c>
-      <c r="F137" s="9" t="s">
+      <c r="F137" s="8" t="s">
         <v>118</v>
       </c>
     </row>
     <row r="138" spans="2:6" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="B138" s="9">
+      <c r="B138" s="8">
         <v>136</v>
       </c>
-      <c r="C138" s="9" t="s">
+      <c r="C138" s="8" t="s">
         <v>271</v>
       </c>
-      <c r="D138" s="9" t="s">
+      <c r="D138" s="8" t="s">
         <v>76</v>
       </c>
-      <c r="E138" s="12">
+      <c r="E138" s="11">
         <v>40303</v>
       </c>
-      <c r="F138" s="9" t="s">
+      <c r="F138" s="8" t="s">
         <v>118</v>
       </c>
     </row>
     <row r="139" spans="2:6" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="B139" s="9">
+      <c r="B139" s="8">
         <v>137</v>
       </c>
-      <c r="C139" s="9" t="s">
+      <c r="C139" s="8" t="s">
         <v>272</v>
       </c>
-      <c r="D139" s="9" t="s">
+      <c r="D139" s="8" t="s">
         <v>76</v>
       </c>
-      <c r="E139" s="12">
+      <c r="E139" s="11">
         <v>40303</v>
       </c>
-      <c r="F139" s="9" t="s">
+      <c r="F139" s="8" t="s">
         <v>118</v>
       </c>
     </row>
     <row r="140" spans="2:6" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="B140" s="9">
+      <c r="B140" s="8">
         <v>138</v>
       </c>
-      <c r="C140" s="9" t="s">
+      <c r="C140" s="8" t="s">
         <v>273</v>
       </c>
-      <c r="D140" s="9" t="s">
+      <c r="D140" s="8" t="s">
         <v>76</v>
       </c>
-      <c r="E140" s="11">
+      <c r="E140" s="10">
         <v>46301</v>
       </c>
-      <c r="F140" s="9" t="s">
+      <c r="F140" s="8" t="s">
         <v>118</v>
       </c>
     </row>
     <row r="141" spans="2:6" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="B141" s="9">
+      <c r="B141" s="8">
         <v>139</v>
       </c>
-      <c r="C141" s="9" t="s">
+      <c r="C141" s="8" t="s">
         <v>274</v>
       </c>
-      <c r="D141" s="9" t="s">
+      <c r="D141" s="8" t="s">
         <v>76</v>
       </c>
-      <c r="E141" s="11">
+      <c r="E141" s="10">
         <v>46301</v>
       </c>
-      <c r="F141" s="9" t="s">
+      <c r="F141" s="8" t="s">
         <v>118</v>
       </c>
     </row>
     <row r="142" spans="2:6" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="B142" s="9">
+      <c r="B142" s="8">
         <v>140</v>
       </c>
-      <c r="C142" s="9" t="s">
+      <c r="C142" s="8" t="s">
         <v>275</v>
       </c>
-      <c r="D142" s="9" t="s">
+      <c r="D142" s="8" t="s">
         <v>76</v>
       </c>
-      <c r="E142" s="11">
+      <c r="E142" s="10">
         <v>46301</v>
       </c>
-      <c r="F142" s="9" t="s">
+      <c r="F142" s="8" t="s">
         <v>118</v>
       </c>
     </row>
     <row r="143" spans="2:6" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="B143" s="9">
+      <c r="B143" s="8">
         <v>141</v>
       </c>
-      <c r="C143" s="9" t="s">
+      <c r="C143" s="8" t="s">
         <v>276</v>
       </c>
-      <c r="D143" s="9" t="s">
+      <c r="D143" s="8" t="s">
         <v>76</v>
       </c>
-      <c r="E143" s="11">
+      <c r="E143" s="10">
         <v>46300</v>
       </c>
-      <c r="F143" s="9" t="s">
+      <c r="F143" s="8" t="s">
         <v>118</v>
       </c>
     </row>
     <row r="144" spans="2:6" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="B144" s="9">
+      <c r="B144" s="8">
         <v>142</v>
       </c>
-      <c r="C144" s="9" t="s">
+      <c r="C144" s="8" t="s">
         <v>277</v>
       </c>
-      <c r="D144" s="9" t="s">
+      <c r="D144" s="8" t="s">
         <v>76</v>
       </c>
-      <c r="E144" s="11">
+      <c r="E144" s="10">
         <v>46301</v>
       </c>
-      <c r="F144" s="9" t="s">
+      <c r="F144" s="8" t="s">
         <v>118</v>
       </c>
     </row>
     <row r="145" spans="2:6" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="B145" s="9">
+      <c r="B145" s="8">
         <v>143</v>
       </c>
-      <c r="C145" s="9" t="s">
+      <c r="C145" s="8" t="s">
         <v>278</v>
       </c>
-      <c r="D145" s="9" t="s">
+      <c r="D145" s="8" t="s">
         <v>76</v>
       </c>
-      <c r="E145" s="11">
+      <c r="E145" s="10">
         <v>46301</v>
       </c>
-      <c r="F145" s="9" t="s">
+      <c r="F145" s="8" t="s">
         <v>118</v>
       </c>
     </row>
     <row r="146" spans="2:6" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="B146" s="9">
+      <c r="B146" s="8">
         <v>144</v>
       </c>
-      <c r="C146" s="9" t="s">
+      <c r="C146" s="8" t="s">
         <v>279</v>
       </c>
-      <c r="D146" s="9" t="s">
+      <c r="D146" s="8" t="s">
         <v>76</v>
       </c>
-      <c r="E146" s="12">
+      <c r="E146" s="11">
         <v>40304</v>
       </c>
-      <c r="F146" s="9" t="s">
+      <c r="F146" s="8" t="s">
         <v>118</v>
       </c>
     </row>
     <row r="147" spans="2:6" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="B147" s="9">
+      <c r="B147" s="8">
         <v>145</v>
       </c>
-      <c r="C147" s="9" t="s">
+      <c r="C147" s="8" t="s">
         <v>280</v>
       </c>
-      <c r="D147" s="9" t="s">
+      <c r="D147" s="8" t="s">
         <v>76</v>
       </c>
-      <c r="E147" s="12">
+      <c r="E147" s="11">
         <v>40304</v>
       </c>
-      <c r="F147" s="9" t="s">
+      <c r="F147" s="8" t="s">
         <v>118</v>
       </c>
     </row>
     <row r="148" spans="2:6" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="B148" s="9">
+      <c r="B148" s="8">
         <v>146</v>
       </c>
-      <c r="C148" s="9" t="s">
+      <c r="C148" s="8" t="s">
         <v>281</v>
       </c>
-      <c r="D148" s="9" t="s">
+      <c r="D148" s="8" t="s">
         <v>76</v>
       </c>
-      <c r="E148" s="12">
+      <c r="E148" s="11">
         <v>40304</v>
       </c>
-      <c r="F148" s="9" t="s">
+      <c r="F148" s="8" t="s">
         <v>118</v>
       </c>
     </row>
     <row r="149" spans="2:6" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="B149" s="9">
+      <c r="B149" s="8">
         <v>147</v>
       </c>
-      <c r="C149" s="9" t="s">
+      <c r="C149" s="8" t="s">
         <v>282</v>
       </c>
-      <c r="D149" s="9" t="s">
+      <c r="D149" s="8" t="s">
         <v>188</v>
       </c>
-      <c r="E149" s="12">
+      <c r="E149" s="11">
         <v>40304</v>
       </c>
-      <c r="F149" s="9" t="s">
+      <c r="F149" s="8" t="s">
         <v>118</v>
       </c>
     </row>
     <row r="150" spans="2:6" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="B150" s="9">
+      <c r="B150" s="8">
         <v>148</v>
       </c>
-      <c r="C150" s="9" t="s">
+      <c r="C150" s="8" t="s">
         <v>283</v>
       </c>
-      <c r="D150" s="9" t="s">
+      <c r="D150" s="8" t="s">
         <v>188</v>
       </c>
-      <c r="E150" s="11">
+      <c r="E150" s="10">
         <v>46301</v>
       </c>
-      <c r="F150" s="9" t="s">
+      <c r="F150" s="8" t="s">
         <v>118</v>
       </c>
     </row>
     <row r="151" spans="2:6" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="B151" s="9">
+      <c r="B151" s="8">
         <v>149</v>
       </c>
-      <c r="C151" s="9" t="s">
+      <c r="C151" s="8" t="s">
         <v>284</v>
       </c>
-      <c r="D151" s="9" t="s">
+      <c r="D151" s="8" t="s">
         <v>188</v>
       </c>
-      <c r="E151" s="11">
+      <c r="E151" s="10">
         <v>46302</v>
       </c>
-      <c r="F151" s="9" t="s">
+      <c r="F151" s="8" t="s">
         <v>285</v>
       </c>
     </row>
     <row r="152" spans="2:6" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="B152" s="9">
+      <c r="B152" s="8">
         <v>150</v>
       </c>
-      <c r="C152" s="9" t="s">
+      <c r="C152" s="8" t="s">
         <v>286</v>
       </c>
-      <c r="D152" s="9" t="s">
+      <c r="D152" s="8" t="s">
         <v>188</v>
       </c>
-      <c r="E152" s="12">
+      <c r="E152" s="11">
         <v>40304</v>
       </c>
-      <c r="F152" s="9" t="s">
+      <c r="F152" s="8" t="s">
         <v>285</v>
       </c>
     </row>
     <row r="153" spans="2:6" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="B153" s="9">
+      <c r="B153" s="8">
         <v>151</v>
       </c>
-      <c r="C153" s="9" t="s">
+      <c r="C153" s="8" t="s">
         <v>287</v>
       </c>
-      <c r="D153" s="9" t="s">
+      <c r="D153" s="8" t="s">
         <v>188</v>
       </c>
-      <c r="E153" s="12">
+      <c r="E153" s="11">
         <v>40304</v>
       </c>
-      <c r="F153" s="9" t="s">
+      <c r="F153" s="8" t="s">
         <v>285</v>
       </c>
     </row>
     <row r="154" spans="2:6" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="B154" s="9">
+      <c r="B154" s="8">
         <v>152</v>
       </c>
-      <c r="C154" s="9" t="s">
+      <c r="C154" s="8" t="s">
         <v>288</v>
       </c>
-      <c r="D154" s="9" t="s">
+      <c r="D154" s="8" t="s">
         <v>188</v>
       </c>
-      <c r="E154" s="12">
+      <c r="E154" s="11">
         <v>40304</v>
       </c>
-      <c r="F154" s="9" t="s">
+      <c r="F154" s="8" t="s">
         <v>285</v>
       </c>
     </row>
     <row r="155" spans="2:6" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="B155" s="9">
+      <c r="B155" s="8">
         <v>153</v>
       </c>
-      <c r="C155" s="9" t="s">
+      <c r="C155" s="8" t="s">
         <v>289</v>
       </c>
-      <c r="D155" s="9" t="s">
+      <c r="D155" s="8" t="s">
         <v>76</v>
       </c>
-      <c r="E155" s="11">
+      <c r="E155" s="10">
         <v>46299</v>
       </c>
-      <c r="F155" s="9" t="s">
+      <c r="F155" s="8" t="s">
         <v>290</v>
       </c>
     </row>
     <row r="156" spans="2:6" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="B156" s="9">
+      <c r="B156" s="8">
         <v>154</v>
       </c>
-      <c r="C156" s="9" t="s">
+      <c r="C156" s="8" t="s">
         <v>291</v>
       </c>
-      <c r="D156" s="9" t="s">
+      <c r="D156" s="8" t="s">
         <v>89</v>
       </c>
-      <c r="E156" s="12">
+      <c r="E156" s="11">
         <v>40301</v>
       </c>
-      <c r="F156" s="9" t="s">
+      <c r="F156" s="8" t="s">
         <v>290</v>
       </c>
     </row>
     <row r="157" spans="2:6" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="B157" s="9">
+      <c r="B157" s="8">
         <v>155</v>
       </c>
-      <c r="C157" s="9" t="s">
+      <c r="C157" s="8" t="s">
         <v>292</v>
       </c>
-      <c r="D157" s="9" t="s">
+      <c r="D157" s="8" t="s">
         <v>64</v>
       </c>
-      <c r="E157" s="12">
+      <c r="E157" s="11">
         <v>40302</v>
       </c>
-      <c r="F157" s="9" t="s">
+      <c r="F157" s="8" t="s">
         <v>293</v>
       </c>
     </row>
     <row r="158" spans="2:6" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="B158" s="9">
+      <c r="B158" s="8">
         <v>156</v>
       </c>
-      <c r="C158" s="9" t="s">
+      <c r="C158" s="8" t="s">
         <v>294</v>
       </c>
-      <c r="D158" s="9" t="s">
+      <c r="D158" s="8" t="s">
         <v>64</v>
       </c>
-      <c r="E158" s="11">
+      <c r="E158" s="10">
         <v>46299</v>
       </c>
-      <c r="F158" s="9" t="s">
+      <c r="F158" s="8" t="s">
         <v>293</v>
       </c>
     </row>
     <row r="159" spans="2:6" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="B159" s="9">
+      <c r="B159" s="8">
         <v>157</v>
       </c>
-      <c r="C159" s="9" t="s">
+      <c r="C159" s="8" t="s">
         <v>295</v>
       </c>
-      <c r="D159" s="9" t="s">
+      <c r="D159" s="8" t="s">
         <v>208</v>
       </c>
-      <c r="E159" s="11">
+      <c r="E159" s="10">
         <v>46299</v>
       </c>
-      <c r="F159" s="9" t="s">
+      <c r="F159" s="8" t="s">
         <v>296</v>
       </c>
     </row>
     <row r="160" spans="2:6" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="B160" s="9">
+      <c r="B160" s="8">
         <v>158</v>
       </c>
-      <c r="C160" s="9" t="s">
+      <c r="C160" s="8" t="s">
         <v>297</v>
       </c>
-      <c r="D160" s="9" t="s">
+      <c r="D160" s="8" t="s">
         <v>64</v>
       </c>
-      <c r="E160" s="11">
+      <c r="E160" s="10">
         <v>46297</v>
       </c>
-      <c r="F160" s="9" t="s">
+      <c r="F160" s="8" t="s">
         <v>298</v>
       </c>
     </row>
     <row r="161" spans="2:6" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="B161" s="9">
+      <c r="B161" s="8">
         <v>159</v>
       </c>
-      <c r="C161" s="9" t="s">
+      <c r="C161" s="8" t="s">
         <v>299</v>
       </c>
-      <c r="D161" s="9" t="s">
+      <c r="D161" s="8" t="s">
         <v>94</v>
       </c>
-      <c r="E161" s="11">
+      <c r="E161" s="10">
         <v>46299</v>
       </c>
-      <c r="F161" s="9" t="s">
+      <c r="F161" s="8" t="s">
         <v>300</v>
       </c>
     </row>
     <row r="162" spans="2:6" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="B162" s="9">
+      <c r="B162" s="8">
         <v>160</v>
       </c>
-      <c r="C162" s="9" t="s">
+      <c r="C162" s="8" t="s">
         <v>301</v>
       </c>
-      <c r="D162" s="9" t="s">
+      <c r="D162" s="8" t="s">
         <v>68</v>
       </c>
-      <c r="E162" s="11">
+      <c r="E162" s="10">
         <v>46300</v>
       </c>
-      <c r="F162" s="9" t="s">
+      <c r="F162" s="8" t="s">
         <v>293</v>
       </c>
     </row>
     <row r="163" spans="2:6" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="B163" s="9">
+      <c r="B163" s="8">
         <v>161</v>
       </c>
-      <c r="C163" s="9" t="s">
+      <c r="C163" s="8" t="s">
         <v>302</v>
       </c>
-      <c r="D163" s="9" t="s">
+      <c r="D163" s="8" t="s">
         <v>76</v>
       </c>
-      <c r="E163" s="11">
+      <c r="E163" s="10">
         <v>46299</v>
       </c>
-      <c r="F163" s="9" t="s">
+      <c r="F163" s="8" t="s">
         <v>303</v>
       </c>
     </row>
     <row r="164" spans="2:6" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="B164" s="9">
+      <c r="B164" s="8">
         <v>162</v>
       </c>
-      <c r="C164" s="9" t="s">
+      <c r="C164" s="8" t="s">
         <v>304</v>
       </c>
-      <c r="D164" s="9" t="s">
+      <c r="D164" s="8" t="s">
         <v>76</v>
       </c>
-      <c r="E164" s="11">
+      <c r="E164" s="10">
         <v>46299</v>
       </c>
-      <c r="F164" s="9" t="s">
+      <c r="F164" s="8" t="s">
         <v>303</v>
       </c>
     </row>
     <row r="165" spans="2:6" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="B165" s="9">
+      <c r="B165" s="8">
         <v>163</v>
       </c>
-      <c r="C165" s="9" t="s">
+      <c r="C165" s="8" t="s">
         <v>305</v>
       </c>
-      <c r="D165" s="9" t="s">
+      <c r="D165" s="8" t="s">
         <v>76</v>
       </c>
-      <c r="E165" s="12">
+      <c r="E165" s="11">
         <v>40304</v>
       </c>
-      <c r="F165" s="9" t="s">
+      <c r="F165" s="8" t="s">
         <v>306</v>
       </c>
     </row>
     <row r="179" spans="2:8" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="B179" s="8" t="s">
+      <c r="B179" s="7" t="s">
         <v>58</v>
       </c>
-      <c r="C179" s="8" t="s">
+      <c r="C179" s="7" t="s">
         <v>361</v>
       </c>
-      <c r="D179" s="8" t="s">
+      <c r="D179" s="7" t="s">
         <v>362</v>
       </c>
-      <c r="E179" s="8" t="s">
+      <c r="E179" s="7" t="s">
         <v>363</v>
       </c>
-      <c r="F179" s="8" t="s">
+      <c r="F179" s="7" t="s">
         <v>364</v>
       </c>
-      <c r="G179" s="8" t="s">
+      <c r="G179" s="7" t="s">
         <v>365</v>
       </c>
-      <c r="H179" s="8" t="s">
+      <c r="H179" s="7" t="s">
         <v>366</v>
       </c>
     </row>
     <row r="180" spans="2:8" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="B180" s="10" t="s">
+      <c r="B180" s="9" t="s">
         <v>367</v>
       </c>
-      <c r="C180" s="9">
+      <c r="C180" s="8">
         <v>9</v>
       </c>
-      <c r="D180" s="9">
+      <c r="D180" s="8">
         <v>10</v>
       </c>
-      <c r="E180" s="9">
+      <c r="E180" s="8">
         <v>9</v>
       </c>
-      <c r="F180" s="9">
+      <c r="F180" s="8">
         <v>10</v>
       </c>
-      <c r="G180" s="9">
+      <c r="G180" s="8">
         <v>8</v>
       </c>
-      <c r="H180" s="10">
+      <c r="H180" s="9">
         <v>9.5</v>
       </c>
     </row>
     <row r="181" spans="2:8" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="B181" s="10" t="s">
+      <c r="B181" s="9" t="s">
         <v>368</v>
       </c>
-      <c r="C181" s="9">
+      <c r="C181" s="8">
         <v>9</v>
       </c>
-      <c r="D181" s="9">
+      <c r="D181" s="8">
         <v>9</v>
       </c>
-      <c r="E181" s="9">
+      <c r="E181" s="8">
         <v>9</v>
       </c>
-      <c r="F181" s="9">
+      <c r="F181" s="8">
         <v>10</v>
       </c>
-      <c r="G181" s="9">
+      <c r="G181" s="8">
         <v>7</v>
       </c>
-      <c r="H181" s="10">
+      <c r="H181" s="9">
         <v>9.1999999999999993</v>
       </c>
     </row>
     <row r="182" spans="2:8" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="B182" s="10" t="s">
+      <c r="B182" s="9" t="s">
         <v>369</v>
       </c>
-      <c r="C182" s="9">
+      <c r="C182" s="8">
         <v>9</v>
       </c>
-      <c r="D182" s="9">
+      <c r="D182" s="8">
         <v>9</v>
       </c>
-      <c r="E182" s="9">
+      <c r="E182" s="8">
         <v>10</v>
       </c>
-      <c r="F182" s="9">
+      <c r="F182" s="8">
         <v>8</v>
       </c>
-      <c r="G182" s="9">
+      <c r="G182" s="8">
         <v>7</v>
       </c>
-      <c r="H182" s="10">
+      <c r="H182" s="9">
         <v>9</v>
       </c>
     </row>
     <row r="183" spans="2:8" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="B183" s="10" t="s">
+      <c r="B183" s="9" t="s">
         <v>370</v>
       </c>
-      <c r="C183" s="9">
+      <c r="C183" s="8">
         <v>8</v>
       </c>
-      <c r="D183" s="9">
+      <c r="D183" s="8">
         <v>8</v>
       </c>
-      <c r="E183" s="9">
+      <c r="E183" s="8">
         <v>9</v>
       </c>
-      <c r="F183" s="9">
+      <c r="F183" s="8">
         <v>10</v>
       </c>
-      <c r="G183" s="9">
+      <c r="G183" s="8">
         <v>8</v>
       </c>
-      <c r="H183" s="10">
+      <c r="H183" s="9">
         <v>8.8000000000000007</v>
       </c>
     </row>
     <row r="184" spans="2:8" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="B184" s="10" t="s">
+      <c r="B184" s="9" t="s">
         <v>371</v>
       </c>
-      <c r="C184" s="9">
+      <c r="C184" s="8">
         <v>8</v>
       </c>
-      <c r="D184" s="9">
+      <c r="D184" s="8">
         <v>9</v>
       </c>
-      <c r="E184" s="9">
+      <c r="E184" s="8">
         <v>8</v>
       </c>
-      <c r="F184" s="9">
+      <c r="F184" s="8">
         <v>9</v>
       </c>
-      <c r="G184" s="9">
+      <c r="G184" s="8">
         <v>7</v>
       </c>
-      <c r="H184" s="10">
+      <c r="H184" s="9">
         <v>8.6999999999999993</v>
       </c>
     </row>
     <row r="185" spans="2:8" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="B185" s="10" t="s">
+      <c r="B185" s="9" t="s">
         <v>372</v>
       </c>
-      <c r="C185" s="9">
+      <c r="C185" s="8">
         <v>7</v>
       </c>
-      <c r="D185" s="9">
+      <c r="D185" s="8">
         <v>9</v>
       </c>
-      <c r="E185" s="9">
+      <c r="E185" s="8">
         <v>8</v>
       </c>
-      <c r="F185" s="9">
+      <c r="F185" s="8">
         <v>8</v>
       </c>
-      <c r="G185" s="9">
+      <c r="G185" s="8">
         <v>9</v>
       </c>
-      <c r="H185" s="10">
+      <c r="H185" s="9">
         <v>8.5</v>
       </c>
     </row>
     <row r="186" spans="2:8" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="B186" s="10" t="s">
+      <c r="B186" s="9" t="s">
         <v>373</v>
       </c>
-      <c r="C186" s="9">
+      <c r="C186" s="8">
         <v>7</v>
       </c>
-      <c r="D186" s="9">
+      <c r="D186" s="8">
         <v>9</v>
       </c>
-      <c r="E186" s="9">
+      <c r="E186" s="8">
         <v>6</v>
       </c>
-      <c r="F186" s="9">
+      <c r="F186" s="8">
         <v>7</v>
       </c>
-      <c r="G186" s="9">
+      <c r="G186" s="8">
         <v>9</v>
       </c>
-      <c r="H186" s="10">
+      <c r="H186" s="9">
         <v>8.3000000000000007</v>
       </c>
     </row>
     <row r="187" spans="2:8" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="B187" s="10" t="s">
+      <c r="B187" s="9" t="s">
         <v>374</v>
       </c>
-      <c r="C187" s="9">
+      <c r="C187" s="8">
         <v>8</v>
       </c>
-      <c r="D187" s="9">
+      <c r="D187" s="8">
         <v>8</v>
       </c>
-      <c r="E187" s="9">
+      <c r="E187" s="8">
         <v>8</v>
       </c>
-      <c r="F187" s="9">
+      <c r="F187" s="8">
         <v>7</v>
       </c>
-      <c r="G187" s="9">
+      <c r="G187" s="8">
         <v>7</v>
       </c>
-      <c r="H187" s="10">
+      <c r="H187" s="9">
         <v>8.1999999999999993</v>
       </c>
     </row>
     <row r="188" spans="2:8" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="B188" s="10" t="s">
+      <c r="B188" s="9" t="s">
         <v>375</v>
       </c>
-      <c r="C188" s="9">
+      <c r="C188" s="8">
         <v>8</v>
       </c>
-      <c r="D188" s="9">
+      <c r="D188" s="8">
         <v>7</v>
       </c>
-      <c r="E188" s="9">
+      <c r="E188" s="8">
         <v>8</v>
       </c>
-      <c r="F188" s="9">
+      <c r="F188" s="8">
         <v>7</v>
       </c>
-      <c r="G188" s="9">
+      <c r="G188" s="8">
         <v>7</v>
       </c>
-      <c r="H188" s="10">
+      <c r="H188" s="9">
         <v>8</v>
       </c>
     </row>
     <row r="189" spans="2:8" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="B189" s="10" t="s">
+      <c r="B189" s="9" t="s">
         <v>376</v>
       </c>
-      <c r="C189" s="9">
+      <c r="C189" s="8">
         <v>7</v>
       </c>
-      <c r="D189" s="9">
+      <c r="D189" s="8">
         <v>8</v>
       </c>
-      <c r="E189" s="9">
+      <c r="E189" s="8">
         <v>7</v>
       </c>
-      <c r="F189" s="9">
+      <c r="F189" s="8">
         <v>7</v>
       </c>
-      <c r="G189" s="9">
+      <c r="G189" s="8">
         <v>7</v>
       </c>
-      <c r="H189" s="10">
+      <c r="H189" s="9">
         <v>7.8</v>
       </c>
     </row>
     <row r="190" spans="2:8" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="B190" s="10" t="s">
+      <c r="B190" s="9" t="s">
         <v>377</v>
       </c>
-      <c r="C190" s="9">
+      <c r="C190" s="8">
         <v>6</v>
       </c>
-      <c r="D190" s="9">
+      <c r="D190" s="8">
         <v>8</v>
       </c>
-      <c r="E190" s="9">
+      <c r="E190" s="8">
         <v>5</v>
       </c>
-      <c r="F190" s="9">
+      <c r="F190" s="8">
         <v>6</v>
       </c>
-      <c r="G190" s="9">
+      <c r="G190" s="8">
         <v>10</v>
       </c>
-      <c r="H190" s="10">
+      <c r="H190" s="9">
         <v>7.6</v>
       </c>
     </row>
     <row r="191" spans="2:8" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="B191" s="10" t="s">
+      <c r="B191" s="9" t="s">
         <v>378</v>
       </c>
-      <c r="C191" s="9">
+      <c r="C191" s="8">
         <v>6</v>
       </c>
-      <c r="D191" s="9">
+      <c r="D191" s="8">
         <v>8</v>
       </c>
-      <c r="E191" s="9">
+      <c r="E191" s="8">
         <v>6</v>
       </c>
-      <c r="F191" s="9">
+      <c r="F191" s="8">
         <v>7</v>
       </c>
-      <c r="G191" s="9">
+      <c r="G191" s="8">
         <v>9</v>
       </c>
-      <c r="H191" s="10">
+      <c r="H191" s="9">
         <v>7.5</v>
       </c>
     </row>
     <row r="192" spans="2:8" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="B192" s="10" t="s">
+      <c r="B192" s="9" t="s">
         <v>379</v>
       </c>
-      <c r="C192" s="9">
+      <c r="C192" s="8">
         <v>7</v>
       </c>
-      <c r="D192" s="9">
+      <c r="D192" s="8">
         <v>7</v>
       </c>
-      <c r="E192" s="9">
+      <c r="E192" s="8">
         <v>7</v>
       </c>
-      <c r="F192" s="9">
+      <c r="F192" s="8">
         <v>6</v>
       </c>
-      <c r="G192" s="9">
+      <c r="G192" s="8">
         <v>7</v>
       </c>
-      <c r="H192" s="10">
+      <c r="H192" s="9">
         <v>7.3</v>
       </c>
     </row>
     <row r="193" spans="2:8" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="B193" s="10" t="s">
+      <c r="B193" s="9" t="s">
         <v>380</v>
       </c>
-      <c r="C193" s="9">
+      <c r="C193" s="8">
         <v>6</v>
       </c>
-      <c r="D193" s="9">
+      <c r="D193" s="8">
         <v>7</v>
       </c>
-      <c r="E193" s="9">
+      <c r="E193" s="8">
         <v>7</v>
       </c>
-      <c r="F193" s="9">
+      <c r="F193" s="8">
         <v>7</v>
       </c>
-      <c r="G193" s="9">
+      <c r="G193" s="8">
         <v>7</v>
       </c>
-      <c r="H193" s="10">
+      <c r="H193" s="9">
         <v>7.2</v>
       </c>
     </row>
     <row r="194" spans="2:8" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="B194" s="10" t="s">
+      <c r="B194" s="9" t="s">
         <v>381</v>
       </c>
-      <c r="C194" s="9">
+      <c r="C194" s="8">
         <v>5</v>
       </c>
-      <c r="D194" s="9">
+      <c r="D194" s="8">
         <v>7</v>
       </c>
-      <c r="E194" s="9">
+      <c r="E194" s="8">
         <v>6</v>
       </c>
-      <c r="F194" s="9">
+      <c r="F194" s="8">
         <v>6</v>
       </c>
-      <c r="G194" s="9">
+      <c r="G194" s="8">
         <v>9</v>
       </c>
-      <c r="H194" s="10">
+      <c r="H194" s="9">
         <v>6.8</v>
       </c>
     </row>
     <row r="195" spans="2:8" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="B195" s="10" t="s">
+      <c r="B195" s="9" t="s">
         <v>382</v>
       </c>
-      <c r="C195" s="9">
+      <c r="C195" s="8">
         <v>6</v>
       </c>
-      <c r="D195" s="9">
+      <c r="D195" s="8">
         <v>6</v>
       </c>
-      <c r="E195" s="9">
+      <c r="E195" s="8">
         <v>6</v>
       </c>
-      <c r="F195" s="9">
+      <c r="F195" s="8">
         <v>5</v>
       </c>
-      <c r="G195" s="9">
+      <c r="G195" s="8">
         <v>7</v>
       </c>
-      <c r="H195" s="10">
+      <c r="H195" s="9">
         <v>6.5</v>
       </c>
     </row>
     <row r="196" spans="2:8" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="B196" s="10" t="s">
+      <c r="B196" s="9" t="s">
         <v>383</v>
       </c>
-      <c r="C196" s="9">
+      <c r="C196" s="8">
         <v>6</v>
       </c>
-      <c r="D196" s="9">
+      <c r="D196" s="8">
         <v>5</v>
       </c>
-      <c r="E196" s="9">
+      <c r="E196" s="8">
         <v>7</v>
       </c>
-      <c r="F196" s="9">
+      <c r="F196" s="8">
         <v>5</v>
       </c>
-      <c r="G196" s="9">
+      <c r="G196" s="8">
         <v>6</v>
       </c>
-      <c r="H196" s="10">
+      <c r="H196" s="9">
         <v>6.3</v>
       </c>
     </row>
     <row r="197" spans="2:8" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="B197" s="10" t="s">
+      <c r="B197" s="9" t="s">
         <v>384</v>
       </c>
-      <c r="C197" s="9">
+      <c r="C197" s="8">
         <v>5</v>
       </c>
-      <c r="D197" s="9">
+      <c r="D197" s="8">
         <v>5</v>
       </c>
-      <c r="E197" s="9">
+      <c r="E197" s="8">
         <v>5</v>
       </c>
-      <c r="F197" s="9">
+      <c r="F197" s="8">
         <v>5</v>
       </c>
-      <c r="G197" s="9">
+      <c r="G197" s="8">
         <v>7</v>
       </c>
-      <c r="H197" s="10">
+      <c r="H197" s="9">
         <v>6</v>
       </c>
     </row>
     <row r="198" spans="2:8" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="B198" s="10" t="s">
+      <c r="B198" s="9" t="s">
         <v>385</v>
       </c>
-      <c r="C198" s="9">
+      <c r="C198" s="8">
         <v>5</v>
       </c>
-      <c r="D198" s="9">
+      <c r="D198" s="8">
         <v>5</v>
       </c>
-      <c r="E198" s="9">
+      <c r="E198" s="8">
         <v>5</v>
       </c>
-      <c r="F198" s="9">
+      <c r="F198" s="8">
         <v>5</v>
       </c>
-      <c r="G198" s="9">
+      <c r="G198" s="8">
         <v>7</v>
       </c>
-      <c r="H198" s="10">
+      <c r="H198" s="9">
         <v>5.8</v>
       </c>
     </row>
     <row r="199" spans="2:8" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="B199" s="10" t="s">
+      <c r="B199" s="9" t="s">
         <v>386</v>
       </c>
-      <c r="C199" s="9">
+      <c r="C199" s="8">
         <v>4</v>
       </c>
-      <c r="D199" s="9">
+      <c r="D199" s="8">
         <v>5</v>
       </c>
-      <c r="E199" s="9">
+      <c r="E199" s="8">
         <v>4</v>
       </c>
-      <c r="F199" s="9">
+      <c r="F199" s="8">
         <v>4</v>
       </c>
-      <c r="G199" s="9">
+      <c r="G199" s="8">
         <v>7</v>
       </c>
-      <c r="H199" s="10">
+      <c r="H199" s="9">
         <v>5.5</v>
       </c>
     </row>
     <row r="202" spans="2:8" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="B202" s="8" t="s">
+      <c r="B202" s="7" t="s">
         <v>57</v>
       </c>
-      <c r="C202" s="8" t="s">
+      <c r="C202" s="7" t="s">
         <v>58</v>
       </c>
-      <c r="D202" s="8" t="s">
+      <c r="D202" s="7" t="s">
         <v>387</v>
       </c>
-      <c r="E202" s="8" t="s">
+      <c r="E202" s="7" t="s">
         <v>388</v>
       </c>
     </row>
     <row r="203" spans="2:8" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="B203" s="9">
+      <c r="B203" s="8">
         <v>1</v>
       </c>
-      <c r="C203" s="10" t="s">
+      <c r="C203" s="9" t="s">
         <v>367</v>
       </c>
-      <c r="D203" s="9" t="s">
+      <c r="D203" s="8" t="s">
         <v>389</v>
       </c>
-      <c r="E203" s="9" t="s">
+      <c r="E203" s="8" t="s">
         <v>390</v>
       </c>
     </row>
     <row r="204" spans="2:8" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="B204" s="9">
+      <c r="B204" s="8">
         <v>2</v>
       </c>
-      <c r="C204" s="10" t="s">
+      <c r="C204" s="9" t="s">
         <v>368</v>
       </c>
-      <c r="D204" s="9" t="s">
+      <c r="D204" s="8" t="s">
         <v>391</v>
       </c>
-      <c r="E204" s="9" t="s">
+      <c r="E204" s="8" t="s">
         <v>392</v>
       </c>
     </row>
     <row r="205" spans="2:8" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="B205" s="9">
+      <c r="B205" s="8">
         <v>3</v>
       </c>
-      <c r="C205" s="10" t="s">
+      <c r="C205" s="9" t="s">
         <v>369</v>
       </c>
-      <c r="D205" s="9" t="s">
+      <c r="D205" s="8" t="s">
         <v>389</v>
       </c>
-      <c r="E205" s="9" t="s">
+      <c r="E205" s="8" t="s">
         <v>393</v>
       </c>
     </row>
     <row r="206" spans="2:8" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="B206" s="9">
+      <c r="B206" s="8">
         <v>4</v>
       </c>
-      <c r="C206" s="10" t="s">
+      <c r="C206" s="9" t="s">
         <v>370</v>
       </c>
-      <c r="D206" s="9" t="s">
+      <c r="D206" s="8" t="s">
         <v>389</v>
       </c>
-      <c r="E206" s="9" t="s">
+      <c r="E206" s="8" t="s">
         <v>394</v>
       </c>
     </row>
     <row r="207" spans="2:8" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="B207" s="9">
+      <c r="B207" s="8">
         <v>5</v>
       </c>
-      <c r="C207" s="10" t="s">
+      <c r="C207" s="9" t="s">
         <v>371</v>
       </c>
-      <c r="D207" s="9" t="s">
+      <c r="D207" s="8" t="s">
         <v>391</v>
       </c>
-      <c r="E207" s="9" t="s">
+      <c r="E207" s="8" t="s">
         <v>395</v>
       </c>
     </row>
     <row r="208" spans="2:8" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="B208" s="9">
+      <c r="B208" s="8">
         <v>6</v>
       </c>
-      <c r="C208" s="10" t="s">
+      <c r="C208" s="9" t="s">
         <v>372</v>
       </c>
-      <c r="D208" s="9" t="s">
+      <c r="D208" s="8" t="s">
         <v>389</v>
       </c>
-      <c r="E208" s="9" t="s">
+      <c r="E208" s="8" t="s">
         <v>396</v>
       </c>
     </row>
     <row r="209" spans="2:5" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="B209" s="9">
+      <c r="B209" s="8">
         <v>7</v>
       </c>
-      <c r="C209" s="10" t="s">
+      <c r="C209" s="9" t="s">
         <v>373</v>
       </c>
-      <c r="D209" s="9" t="s">
+      <c r="D209" s="8" t="s">
         <v>389</v>
       </c>
-      <c r="E209" s="9" t="s">
+      <c r="E209" s="8" t="s">
         <v>397</v>
       </c>
     </row>
     <row r="210" spans="2:5" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="B210" s="9">
+      <c r="B210" s="8">
         <v>8</v>
       </c>
-      <c r="C210" s="10" t="s">
+      <c r="C210" s="9" t="s">
         <v>374</v>
       </c>
-      <c r="D210" s="9" t="s">
+      <c r="D210" s="8" t="s">
         <v>391</v>
       </c>
-      <c r="E210" s="9" t="s">
+      <c r="E210" s="8" t="s">
         <v>398</v>
       </c>
     </row>
     <row r="211" spans="2:5" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="B211" s="9">
+      <c r="B211" s="8">
         <v>9</v>
       </c>
-      <c r="C211" s="10" t="s">
+      <c r="C211" s="9" t="s">
         <v>378</v>
       </c>
-      <c r="D211" s="9" t="s">
+      <c r="D211" s="8" t="s">
         <v>391</v>
       </c>
-      <c r="E211" s="9" t="s">
+      <c r="E211" s="8" t="s">
         <v>399</v>
       </c>
     </row>
     <row r="212" spans="2:5" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="B212" s="9">
+      <c r="B212" s="8">
         <v>10</v>
       </c>
-      <c r="C212" s="10" t="s">
+      <c r="C212" s="9" t="s">
         <v>379</v>
       </c>
-      <c r="D212" s="9" t="s">
+      <c r="D212" s="8" t="s">
         <v>391</v>
       </c>
-      <c r="E212" s="9" t="s">
+      <c r="E212" s="8" t="s">
         <v>400</v>
       </c>
     </row>
     <row r="213" spans="2:5" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="B213" s="9">
+      <c r="B213" s="8">
         <v>11</v>
       </c>
-      <c r="C213" s="10" t="s">
+      <c r="C213" s="9" t="s">
         <v>377</v>
       </c>
-      <c r="D213" s="9" t="s">
+      <c r="D213" s="8" t="s">
         <v>389</v>
       </c>
-      <c r="E213" s="9" t="s">
+      <c r="E213" s="8" t="s">
         <v>401</v>
       </c>
     </row>

</xml_diff>

<commit_message>
start try fix zz problems
</commit_message>
<xml_diff>
--- a/__docs/RoadMap.xlsx
+++ b/__docs/RoadMap.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Dev\exchange\RichLaughter3\__docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2599BF5F-40A2-4746-928B-BF847809B95F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CBE2DF6D-F275-4A65-9F69-C0C1698BAD0A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Тезисы" sheetId="1" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="957" uniqueCount="433">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="961" uniqueCount="435">
   <si>
     <t>RL3 - это продолжение RL1</t>
   </si>
@@ -1363,6 +1363,12 @@
   </si>
   <si>
     <t>Адаптация из RL1. Логика отличается</t>
+  </si>
+  <si>
+    <t>PEG19_JOHANNA</t>
+  </si>
+  <si>
+    <t>FixVanga Problem - когда после смещения будущего теряются актуальные данные</t>
   </si>
 </sst>
 </file>
@@ -1443,7 +1449,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1475,6 +1481,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="14" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Обычный" xfId="0" builtinId="0"/>
@@ -5049,7 +5056,7 @@
       </c>
       <c r="L2">
         <f>COUNTIF(D:D,L1)</f>
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="M2">
         <f>COUNTIF(D:D,M1)</f>
@@ -6200,16 +6207,16 @@
       <c r="A69">
         <v>68</v>
       </c>
-      <c r="B69" t="s">
+      <c r="B69" s="6" t="s">
         <v>358</v>
       </c>
-      <c r="C69" s="3">
+      <c r="C69" s="13">
         <v>46249</v>
       </c>
-      <c r="D69" t="s">
+      <c r="D69" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="E69" t="s">
+      <c r="E69" s="6" t="s">
         <v>44</v>
       </c>
     </row>
@@ -6217,16 +6224,16 @@
       <c r="A70">
         <v>69</v>
       </c>
-      <c r="B70" t="s">
+      <c r="B70" s="6" t="s">
         <v>359</v>
       </c>
-      <c r="C70" s="3">
+      <c r="C70" s="13">
         <v>46249</v>
       </c>
-      <c r="D70" t="s">
+      <c r="D70" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="E70" t="s">
+      <c r="E70" s="6" t="s">
         <v>44</v>
       </c>
     </row>
@@ -6234,16 +6241,16 @@
       <c r="A71">
         <v>70</v>
       </c>
-      <c r="B71" t="s">
+      <c r="B71" s="6" t="s">
         <v>360</v>
       </c>
-      <c r="C71" s="3">
+      <c r="C71" s="13">
         <v>46249</v>
       </c>
-      <c r="D71" t="s">
+      <c r="D71" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="E71" t="s">
+      <c r="E71" s="6" t="s">
         <v>44</v>
       </c>
     </row>
@@ -6261,7 +6268,7 @@
         <v>12</v>
       </c>
       <c r="E72" t="s">
-        <v>44</v>
+        <v>432</v>
       </c>
     </row>
     <row r="73" spans="1:5" x14ac:dyDescent="0.25">
@@ -6278,7 +6285,7 @@
         <v>12</v>
       </c>
       <c r="E73" t="s">
-        <v>44</v>
+        <v>432</v>
       </c>
     </row>
     <row r="74" spans="1:5" x14ac:dyDescent="0.25">
@@ -6295,7 +6302,7 @@
         <v>12</v>
       </c>
       <c r="E74" t="s">
-        <v>44</v>
+        <v>432</v>
       </c>
     </row>
     <row r="75" spans="1:5" x14ac:dyDescent="0.25">
@@ -6312,7 +6319,7 @@
         <v>12</v>
       </c>
       <c r="E75" t="s">
-        <v>44</v>
+        <v>432</v>
       </c>
     </row>
     <row r="76" spans="1:5" x14ac:dyDescent="0.25">
@@ -6431,7 +6438,7 @@
         <v>12</v>
       </c>
       <c r="E82" t="s">
-        <v>44</v>
+        <v>432</v>
       </c>
     </row>
     <row r="83" spans="1:5" x14ac:dyDescent="0.25">
@@ -6726,6 +6733,18 @@
     <row r="100" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A100">
         <v>99</v>
+      </c>
+      <c r="B100" t="s">
+        <v>433</v>
+      </c>
+      <c r="C100" s="3">
+        <v>46252</v>
+      </c>
+      <c r="D100" t="s">
+        <v>12</v>
+      </c>
+      <c r="E100" t="s">
+        <v>44</v>
       </c>
     </row>
     <row r="101" spans="1:5" x14ac:dyDescent="0.25">
@@ -8227,7 +8246,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D5C6E19E-FDB9-4B9E-B0A7-1D91E81DACEB}">
-  <dimension ref="A2:B5"/>
+  <dimension ref="A2:B6"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
@@ -8260,6 +8279,14 @@
       </c>
       <c r="B5" t="s">
         <v>430</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A6">
+        <v>5</v>
+      </c>
+      <c r="B6" t="s">
+        <v>434</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
try resolve zz problems
</commit_message>
<xml_diff>
--- a/__docs/RoadMap.xlsx
+++ b/__docs/RoadMap.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Dev\exchange\RichLaughter3\__docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CBE2DF6D-F275-4A65-9F69-C0C1698BAD0A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3FE73BD1-BF09-4F24-81F6-7E149CD70031}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Тезисы" sheetId="1" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="961" uniqueCount="435">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="964" uniqueCount="437">
   <si>
     <t>RL3 - это продолжение RL1</t>
   </si>
@@ -1369,6 +1369,12 @@
   </si>
   <si>
     <t>FixVanga Problem - когда после смещения будущего теряются актуальные данные</t>
+  </si>
+  <si>
+    <t>PEG22_SONYA</t>
+  </si>
+  <si>
+    <t>PEG22_BERSERK с percent_zz</t>
   </si>
 </sst>
 </file>
@@ -1478,10 +1484,10 @@
     <xf numFmtId="14" fontId="4" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1" indent="1"/>
     </xf>
+    <xf numFmtId="14" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="14" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Обычный" xfId="0" builtinId="0"/>
@@ -1815,7 +1821,7 @@
       </c>
     </row>
     <row r="3" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B3" s="12" t="s">
+      <c r="B3" s="13" t="s">
         <v>3</v>
       </c>
       <c r="C3" s="2" t="s">
@@ -1823,13 +1829,13 @@
       </c>
     </row>
     <row r="4" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B4" s="12"/>
+      <c r="B4" s="13"/>
       <c r="C4" s="2" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="5" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B5" s="12" t="s">
+      <c r="B5" s="13" t="s">
         <v>4</v>
       </c>
       <c r="C5" s="2" t="s">
@@ -1837,43 +1843,43 @@
       </c>
     </row>
     <row r="6" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B6" s="12"/>
+      <c r="B6" s="13"/>
       <c r="C6" s="2" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="7" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B7" s="12"/>
+      <c r="B7" s="13"/>
       <c r="C7" s="2" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="8" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B8" s="12"/>
+      <c r="B8" s="13"/>
       <c r="C8" s="2" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="9" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B9" s="12"/>
+      <c r="B9" s="13"/>
       <c r="C9" s="2" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="10" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B10" s="12"/>
+      <c r="B10" s="13"/>
       <c r="C10" s="2" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="11" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B11" s="12"/>
+      <c r="B11" s="13"/>
       <c r="C11" s="2" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="12" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B12" s="12"/>
+      <c r="B12" s="13"/>
       <c r="C12" s="2" t="s">
         <v>17</v>
       </c>
@@ -5056,7 +5062,7 @@
       </c>
       <c r="L2">
         <f>COUNTIF(D:D,L1)</f>
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="M2">
         <f>COUNTIF(D:D,M1)</f>
@@ -6210,7 +6216,7 @@
       <c r="B69" s="6" t="s">
         <v>358</v>
       </c>
-      <c r="C69" s="13">
+      <c r="C69" s="12">
         <v>46249</v>
       </c>
       <c r="D69" s="6" t="s">
@@ -6227,7 +6233,7 @@
       <c r="B70" s="6" t="s">
         <v>359</v>
       </c>
-      <c r="C70" s="13">
+      <c r="C70" s="12">
         <v>46249</v>
       </c>
       <c r="D70" s="6" t="s">
@@ -6244,7 +6250,7 @@
       <c r="B71" s="6" t="s">
         <v>360</v>
       </c>
-      <c r="C71" s="13">
+      <c r="C71" s="12">
         <v>46249</v>
       </c>
       <c r="D71" s="6" t="s">
@@ -6455,7 +6461,7 @@
         <v>12</v>
       </c>
       <c r="E83" t="s">
-        <v>44</v>
+        <v>432</v>
       </c>
     </row>
     <row r="84" spans="1:5" x14ac:dyDescent="0.25">
@@ -6472,7 +6478,7 @@
         <v>12</v>
       </c>
       <c r="E84" t="s">
-        <v>44</v>
+        <v>432</v>
       </c>
     </row>
     <row r="85" spans="1:5" x14ac:dyDescent="0.25">
@@ -6489,7 +6495,7 @@
         <v>12</v>
       </c>
       <c r="E85" t="s">
-        <v>44</v>
+        <v>432</v>
       </c>
     </row>
     <row r="86" spans="1:5" x14ac:dyDescent="0.25">
@@ -6750,6 +6756,18 @@
     <row r="101" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A101">
         <v>100</v>
+      </c>
+      <c r="B101" t="s">
+        <v>435</v>
+      </c>
+      <c r="C101" s="3">
+        <v>46253</v>
+      </c>
+      <c r="D101" t="s">
+        <v>12</v>
+      </c>
+      <c r="E101" t="s">
+        <v>436</v>
       </c>
     </row>
     <row r="102" spans="1:5" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
new PEG18 with st
</commit_message>
<xml_diff>
--- a/__docs/RoadMap.xlsx
+++ b/__docs/RoadMap.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Dev\exchange\RichLaughter3\__docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{22971122-7A3C-4657-8E5D-71E9DB64BAB1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A654296A-BAA3-4553-BECB-58D167CF9200}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,6 +20,7 @@
     <sheet name="ДрРоботов" sheetId="5" r:id="rId5"/>
     <sheet name="ТекПроблем" sheetId="6" r:id="rId6"/>
     <sheet name="Анализ нейронки стратегий" sheetId="7" r:id="rId7"/>
+    <sheet name="Работа" sheetId="8" r:id="rId8"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -40,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="967" uniqueCount="439">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1000" uniqueCount="453">
   <si>
     <t>RL3 - это продолжение RL1</t>
   </si>
@@ -1381,6 +1382,48 @@
   </si>
   <si>
     <t>Вариативный WEG3_DS</t>
+  </si>
+  <si>
+    <t>Что делал</t>
+  </si>
+  <si>
+    <t>Своб</t>
+  </si>
+  <si>
+    <t>PEG18 на супертренде</t>
+  </si>
+  <si>
+    <t>PEG18_REXXAR2</t>
+  </si>
+  <si>
+    <t>PEG18_UTER2</t>
+  </si>
+  <si>
+    <t>PEG18 на супертренде с дополнительными улучшениями</t>
+  </si>
+  <si>
+    <t>PEG18_DIABLO2</t>
+  </si>
+  <si>
+    <t>Дата удаления</t>
+  </si>
+  <si>
+    <t>PEG18_VARIAN2</t>
+  </si>
+  <si>
+    <t>PEG18_ANDUIN</t>
+  </si>
+  <si>
+    <t>PEG18_VARIAN2 на adx</t>
+  </si>
+  <si>
+    <t>Батя может симулировать</t>
+  </si>
+  <si>
+    <t>Причина удаления</t>
+  </si>
+  <si>
+    <t>add_pc_stair_fast слишком Mcfly</t>
   </si>
 </sst>
 </file>
@@ -5017,7 +5060,9 @@
     <col min="2" max="2" width="21.5703125" customWidth="1"/>
     <col min="3" max="3" width="14" customWidth="1"/>
     <col min="4" max="4" width="7.28515625" customWidth="1"/>
-    <col min="5" max="5" width="44.85546875" customWidth="1"/>
+    <col min="5" max="5" width="55" customWidth="1"/>
+    <col min="6" max="6" width="13.85546875" customWidth="1"/>
+    <col min="7" max="7" width="31.28515625" customWidth="1"/>
     <col min="11" max="11" width="14.5703125" customWidth="1"/>
   </cols>
   <sheetData>
@@ -5034,6 +5079,12 @@
       <c r="E1" t="s">
         <v>27</v>
       </c>
+      <c r="F1" t="s">
+        <v>446</v>
+      </c>
+      <c r="G1" t="s">
+        <v>451</v>
+      </c>
       <c r="L1" t="s">
         <v>12</v>
       </c>
@@ -5068,7 +5119,7 @@
       </c>
       <c r="L2">
         <f>COUNTIF(D:D,L1)</f>
-        <v>42</v>
+        <v>47</v>
       </c>
       <c r="M2">
         <f>COUNTIF(D:D,M1)</f>
@@ -5120,7 +5171,7 @@
       <c r="E4" t="s">
         <v>31</v>
       </c>
-      <c r="F4" t="s">
+      <c r="H4" t="s">
         <v>37</v>
       </c>
     </row>
@@ -5140,7 +5191,7 @@
       <c r="E5" t="s">
         <v>32</v>
       </c>
-      <c r="F5" t="s">
+      <c r="H5" t="s">
         <v>38</v>
       </c>
     </row>
@@ -5603,7 +5654,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A33">
         <v>32</v>
       </c>
@@ -5619,8 +5670,14 @@
       <c r="E33" t="s">
         <v>44</v>
       </c>
-    </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F33" s="3">
+        <v>46266</v>
+      </c>
+      <c r="G33" t="s">
+        <v>450</v>
+      </c>
+    </row>
+    <row r="34" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A34">
         <v>33</v>
       </c>
@@ -5637,7 +5694,7 @@
         <v>432</v>
       </c>
     </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A35">
         <v>34</v>
       </c>
@@ -5654,7 +5711,7 @@
         <v>432</v>
       </c>
     </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A36">
         <v>35</v>
       </c>
@@ -5671,7 +5728,7 @@
         <v>432</v>
       </c>
     </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A37">
         <v>36</v>
       </c>
@@ -5688,7 +5745,7 @@
         <v>432</v>
       </c>
     </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A38">
         <v>37</v>
       </c>
@@ -5705,7 +5762,7 @@
         <v>432</v>
       </c>
     </row>
-    <row r="39" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A39">
         <v>38</v>
       </c>
@@ -5722,7 +5779,7 @@
         <v>432</v>
       </c>
     </row>
-    <row r="40" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A40">
         <v>39</v>
       </c>
@@ -5739,7 +5796,7 @@
         <v>432</v>
       </c>
     </row>
-    <row r="41" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A41">
         <v>40</v>
       </c>
@@ -5756,7 +5813,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="42" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A42">
         <v>41</v>
       </c>
@@ -5773,7 +5830,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="43" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A43">
         <v>42</v>
       </c>
@@ -5790,7 +5847,7 @@
         <v>432</v>
       </c>
     </row>
-    <row r="44" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A44">
         <v>43</v>
       </c>
@@ -5807,7 +5864,7 @@
         <v>432</v>
       </c>
     </row>
-    <row r="45" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A45">
         <v>44</v>
       </c>
@@ -5824,7 +5881,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="46" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A46">
         <v>45</v>
       </c>
@@ -5841,7 +5898,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="47" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A47">
         <v>46</v>
       </c>
@@ -5858,7 +5915,7 @@
         <v>432</v>
       </c>
     </row>
-    <row r="48" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A48">
         <v>47</v>
       </c>
@@ -6147,7 +6204,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="65" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A65">
         <v>64</v>
       </c>
@@ -6164,7 +6221,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="66" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A66">
         <v>65</v>
       </c>
@@ -6181,7 +6238,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="67" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A67">
         <v>66</v>
       </c>
@@ -6198,7 +6255,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="68" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A68">
         <v>67</v>
       </c>
@@ -6215,7 +6272,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="69" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A69">
         <v>68</v>
       </c>
@@ -6232,7 +6289,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="70" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A70">
         <v>69</v>
       </c>
@@ -6249,7 +6306,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="71" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A71">
         <v>70</v>
       </c>
@@ -6266,7 +6323,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="72" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A72">
         <v>71</v>
       </c>
@@ -6282,8 +6339,14 @@
       <c r="E72" t="s">
         <v>432</v>
       </c>
-    </row>
-    <row r="73" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F72" s="3">
+        <v>46266</v>
+      </c>
+      <c r="G72" t="s">
+        <v>452</v>
+      </c>
+    </row>
+    <row r="73" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A73">
         <v>72</v>
       </c>
@@ -6300,7 +6363,7 @@
         <v>432</v>
       </c>
     </row>
-    <row r="74" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A74">
         <v>73</v>
       </c>
@@ -6316,8 +6379,14 @@
       <c r="E74" t="s">
         <v>432</v>
       </c>
-    </row>
-    <row r="75" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F74" s="3">
+        <v>46266</v>
+      </c>
+      <c r="G74" t="s">
+        <v>452</v>
+      </c>
+    </row>
+    <row r="75" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A75">
         <v>74</v>
       </c>
@@ -6333,8 +6402,14 @@
       <c r="E75" t="s">
         <v>432</v>
       </c>
-    </row>
-    <row r="76" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F75" s="3">
+        <v>46266</v>
+      </c>
+      <c r="G75" t="s">
+        <v>452</v>
+      </c>
+    </row>
+    <row r="76" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A76">
         <v>75</v>
       </c>
@@ -6351,7 +6426,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="77" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A77">
         <v>76</v>
       </c>
@@ -6368,7 +6443,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="78" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A78">
         <v>77</v>
       </c>
@@ -6385,7 +6460,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="79" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A79">
         <v>78</v>
       </c>
@@ -6402,7 +6477,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="80" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A80">
         <v>79</v>
       </c>
@@ -6797,25 +6872,85 @@
       <c r="A103">
         <v>102</v>
       </c>
+      <c r="B103" t="s">
+        <v>442</v>
+      </c>
+      <c r="C103" s="3">
+        <v>46266</v>
+      </c>
+      <c r="D103" t="s">
+        <v>12</v>
+      </c>
+      <c r="E103" t="s">
+        <v>441</v>
+      </c>
     </row>
     <row r="104" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A104">
         <v>103</v>
       </c>
+      <c r="B104" t="s">
+        <v>443</v>
+      </c>
+      <c r="C104" s="3">
+        <v>46266</v>
+      </c>
+      <c r="D104" t="s">
+        <v>12</v>
+      </c>
+      <c r="E104" t="s">
+        <v>444</v>
+      </c>
     </row>
     <row r="105" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A105">
         <v>104</v>
       </c>
+      <c r="B105" t="s">
+        <v>445</v>
+      </c>
+      <c r="C105" s="3">
+        <v>46266</v>
+      </c>
+      <c r="D105" t="s">
+        <v>12</v>
+      </c>
+      <c r="E105" t="s">
+        <v>441</v>
+      </c>
     </row>
     <row r="106" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A106">
         <v>105</v>
       </c>
+      <c r="B106" t="s">
+        <v>447</v>
+      </c>
+      <c r="C106" s="3">
+        <v>46266</v>
+      </c>
+      <c r="D106" t="s">
+        <v>12</v>
+      </c>
+      <c r="E106" t="s">
+        <v>441</v>
+      </c>
     </row>
     <row r="107" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A107">
         <v>106</v>
+      </c>
+      <c r="B107" t="s">
+        <v>448</v>
+      </c>
+      <c r="C107" s="3">
+        <v>46266</v>
+      </c>
+      <c r="D107" t="s">
+        <v>12</v>
+      </c>
+      <c r="E107" t="s">
+        <v>449</v>
       </c>
     </row>
     <row r="108" spans="1:5" x14ac:dyDescent="0.25">
@@ -11975,4 +12110,82 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CD57C989-6F2B-410E-8934-538033C06A98}">
+  <dimension ref="A1:D11"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="3" max="3" width="10.5703125" customWidth="1"/>
+    <col min="4" max="4" width="43.42578125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="C1" t="s">
+        <v>25</v>
+      </c>
+      <c r="D1" t="s">
+        <v>439</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A2">
+        <v>1</v>
+      </c>
+      <c r="B2" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="B3" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="B4" t="s">
+        <v>12</v>
+      </c>
+      <c r="C4" s="3">
+        <v>46266</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="B5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="B6" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="B7" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="B8" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="B9" t="s">
+        <v>440</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="B10" t="s">
+        <v>440</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="B11" t="s">
+        <v>440</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>